<commit_message>
Small fix - add 1 DEC
</commit_message>
<xml_diff>
--- a/curation/draft/cdisc_biomedical_concepts_r16_draft.xlsx
+++ b/curation/draft/cdisc_biomedical_concepts_r16_draft.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BC Hierarchy" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Biomedical Concepts'!$A$1:$Q$576</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Biomedical Concepts'!$A$1:$Q$577</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'BC Hierarchy'!$A$1:$K$1</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1" concurrentCalc="0"/>
@@ -839,7 +839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q576"/>
+  <dimension ref="A1:Q577"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.42578125" defaultRowHeight="12" customHeight="1"/>
   <cols>
     <col width="15.7109375" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -35337,22 +35337,22 @@
       <c r="L464" s="20" t="inlineStr"/>
       <c r="M464" s="20" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="N464" s="22" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="O464" s="20" t="inlineStr">
         <is>
-          <t>Collection Date Time</t>
+          <t>Observation Result</t>
         </is>
       </c>
       <c r="P464" s="20" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="Q464" s="21" t="inlineStr"/>
@@ -35408,22 +35408,22 @@
       <c r="L465" s="20" t="inlineStr"/>
       <c r="M465" s="20" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="N465" s="22" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="O465" s="20" t="inlineStr">
         <is>
-          <t>Observation Result</t>
+          <t>Collection Date Time</t>
         </is>
       </c>
       <c r="P465" s="20" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="Q465" s="21" t="inlineStr"/>
@@ -35479,25 +35479,29 @@
       <c r="L466" s="20" t="inlineStr"/>
       <c r="M466" s="20" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C48570</t>
         </is>
       </c>
       <c r="N466" s="22" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C48570</t>
         </is>
       </c>
       <c r="O466" s="20" t="inlineStr">
         <is>
-          <t>Observation Result</t>
+          <t>Percent Unit</t>
         </is>
       </c>
       <c r="P466" s="20" t="inlineStr">
         <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="Q466" s="21" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="Q466" s="21" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
     </row>
     <row r="467">
       <c r="A467" s="20" t="inlineStr">
@@ -35550,29 +35554,25 @@
       <c r="L467" s="20" t="inlineStr"/>
       <c r="M467" s="20" t="inlineStr">
         <is>
-          <t>C48570</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="N467" s="22" t="inlineStr">
         <is>
-          <t>C48570</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="O467" s="20" t="inlineStr">
         <is>
-          <t>Percent Unit</t>
+          <t>Collection Date Time</t>
         </is>
       </c>
       <c r="P467" s="20" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="Q467" s="21" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
+          <t>datetime</t>
+        </is>
+      </c>
+      <c r="Q467" s="21" t="inlineStr"/>
     </row>
     <row r="468">
       <c r="A468" s="20" t="inlineStr">
@@ -35625,22 +35625,22 @@
       <c r="L468" s="20" t="inlineStr"/>
       <c r="M468" s="20" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="N468" s="22" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="O468" s="20" t="inlineStr">
         <is>
-          <t>Collection Date Time</t>
+          <t>Observation Result</t>
         </is>
       </c>
       <c r="P468" s="20" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="Q468" s="21" t="inlineStr"/>
@@ -36059,25 +36059,29 @@
       <c r="L474" s="20" t="inlineStr"/>
       <c r="M474" s="20" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C44276</t>
         </is>
       </c>
       <c r="N474" s="22" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C44276</t>
         </is>
       </c>
       <c r="O474" s="20" t="inlineStr">
         <is>
-          <t>Observation Result</t>
+          <t>Unit of Temperature</t>
         </is>
       </c>
       <c r="P474" s="20" t="inlineStr">
         <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="Q474" s="21" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="Q474" s="21" t="inlineStr">
+        <is>
+          <t>C;F</t>
+        </is>
+      </c>
     </row>
     <row r="475">
       <c r="A475" s="20" t="inlineStr">
@@ -36130,29 +36134,25 @@
       <c r="L475" s="20" t="inlineStr"/>
       <c r="M475" s="20" t="inlineStr">
         <is>
-          <t>C44276</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="N475" s="22" t="inlineStr">
         <is>
-          <t>C44276</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="O475" s="20" t="inlineStr">
         <is>
-          <t>Unit of Temperature</t>
+          <t>Observation Result</t>
         </is>
       </c>
       <c r="P475" s="20" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="Q475" s="21" t="inlineStr">
-        <is>
-          <t>C;F</t>
-        </is>
-      </c>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="Q475" s="21" t="inlineStr"/>
     </row>
     <row r="476">
       <c r="A476" s="20" t="inlineStr">
@@ -36252,29 +36252,25 @@
       <c r="L477" s="20" t="inlineStr"/>
       <c r="M477" s="20" t="inlineStr">
         <is>
-          <t>C82535</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="N477" s="22" t="inlineStr">
         <is>
-          <t>C82535</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="O477" s="20" t="inlineStr">
         <is>
-          <t>Test Method</t>
+          <t>Collection Date Time</t>
         </is>
       </c>
       <c r="P477" s="20" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="Q477" s="21" t="inlineStr">
-        <is>
-          <t>X-Ray;CT Scan</t>
-        </is>
-      </c>
+          <t>datetime</t>
+        </is>
+      </c>
+      <c r="Q477" s="21" t="inlineStr"/>
     </row>
     <row r="478">
       <c r="A478" s="20" t="inlineStr">
@@ -36327,17 +36323,17 @@
       <c r="L478" s="20" t="inlineStr"/>
       <c r="M478" s="20" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82535</t>
         </is>
       </c>
       <c r="N478" s="22" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82535</t>
         </is>
       </c>
       <c r="O478" s="20" t="inlineStr">
         <is>
-          <t>Observation Result</t>
+          <t>Test Method</t>
         </is>
       </c>
       <c r="P478" s="20" t="inlineStr">
@@ -36347,7 +36343,7 @@
       </c>
       <c r="Q478" s="21" t="inlineStr">
         <is>
-          <t>U;N;Y</t>
+          <t>X-Ray;CT Scan</t>
         </is>
       </c>
     </row>
@@ -36359,44 +36355,72 @@
       </c>
       <c r="B479" s="21" t="inlineStr">
         <is>
-          <t>Pulmonary Function Test</t>
+          <t>Pneumonia Indicator</t>
         </is>
       </c>
       <c r="C479" s="20" t="inlineStr">
         <is>
-          <t>C38081</t>
+          <t>C171521</t>
         </is>
       </c>
       <c r="D479" s="22" t="inlineStr">
         <is>
-          <t>C38081</t>
-        </is>
-      </c>
-      <c r="E479" s="20" t="n"/>
+          <t>C171521</t>
+        </is>
+      </c>
+      <c r="E479" s="22" t="inlineStr">
+        <is>
+          <t>C181043</t>
+        </is>
+      </c>
       <c r="F479" s="21" t="inlineStr">
         <is>
-          <t>Respiratory System Findings;Pulmonary Function Tests;Vital Signs</t>
+          <t>Clinical Findings Indicators;Respiratory System Findings</t>
         </is>
       </c>
       <c r="G479" s="20" t="inlineStr">
         <is>
-          <t>Pulmonary Function Test;lung function test;PFT;Pulmonary Function Testing</t>
-        </is>
-      </c>
-      <c r="H479" s="20" t="inlineStr"/>
+          <t>PNEUMIND</t>
+        </is>
+      </c>
+      <c r="H479" s="20" t="inlineStr">
+        <is>
+          <t>Nominal</t>
+        </is>
+      </c>
       <c r="I479" s="21" t="inlineStr">
         <is>
-          <t>A broad range of tests that are performed to assess how well lungs inhale and exhale air and how efficiently they transfer oxygen into the blood.</t>
+          <t>An indication as to whether pneumonia has occurred.</t>
         </is>
       </c>
       <c r="J479" s="20" t="inlineStr"/>
       <c r="K479" s="20" t="inlineStr"/>
       <c r="L479" s="20" t="inlineStr"/>
-      <c r="M479" s="20" t="inlineStr"/>
-      <c r="N479" s="20" t="n"/>
-      <c r="O479" s="20" t="inlineStr"/>
-      <c r="P479" s="20" t="inlineStr"/>
-      <c r="Q479" s="21" t="inlineStr"/>
+      <c r="M479" s="20" t="inlineStr">
+        <is>
+          <t>C70856</t>
+        </is>
+      </c>
+      <c r="N479" s="22" t="inlineStr">
+        <is>
+          <t>C70856</t>
+        </is>
+      </c>
+      <c r="O479" s="20" t="inlineStr">
+        <is>
+          <t>Observation Result</t>
+        </is>
+      </c>
+      <c r="P479" s="20" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="Q479" s="21" t="inlineStr">
+        <is>
+          <t>U;N;Y</t>
+        </is>
+      </c>
     </row>
     <row r="480">
       <c r="A480" s="20" t="inlineStr">
@@ -36406,67 +36430,43 @@
       </c>
       <c r="B480" s="21" t="inlineStr">
         <is>
-          <t>Pulmonary Inertance</t>
+          <t>Pulmonary Function Test</t>
         </is>
       </c>
       <c r="C480" s="20" t="inlineStr">
         <is>
-          <t>C139254</t>
+          <t>C38081</t>
         </is>
       </c>
       <c r="D480" s="22" t="inlineStr">
         <is>
-          <t>C139254</t>
-        </is>
-      </c>
-      <c r="E480" s="22" t="inlineStr">
-        <is>
           <t>C38081</t>
         </is>
       </c>
+      <c r="E480" s="20" t="n"/>
       <c r="F480" s="21" t="inlineStr">
         <is>
-          <t>Respiratory System Findings;Pulmonary Function Test</t>
+          <t>Respiratory System Findings;Pulmonary Function Tests;Vital Signs</t>
         </is>
       </c>
       <c r="G480" s="20" t="inlineStr">
         <is>
-          <t>INERTANC;Inertance</t>
-        </is>
-      </c>
-      <c r="H480" s="20" t="inlineStr">
-        <is>
-          <t>Quantitative</t>
-        </is>
-      </c>
+          <t>Pulmonary Function Test;lung function test;PFT;Pulmonary Function Testing</t>
+        </is>
+      </c>
+      <c r="H480" s="20" t="inlineStr"/>
       <c r="I480" s="21" t="inlineStr">
         <is>
-          <t>The measure of the force of the column of air in the conducting airways.</t>
+          <t>A broad range of tests that are performed to assess how well lungs inhale and exhale air and how efficiently they transfer oxygen into the blood.</t>
         </is>
       </c>
       <c r="J480" s="20" t="inlineStr"/>
       <c r="K480" s="20" t="inlineStr"/>
       <c r="L480" s="20" t="inlineStr"/>
-      <c r="M480" s="20" t="inlineStr">
-        <is>
-          <t>C70856</t>
-        </is>
-      </c>
-      <c r="N480" s="22" t="inlineStr">
-        <is>
-          <t>C70856</t>
-        </is>
-      </c>
-      <c r="O480" s="20" t="inlineStr">
-        <is>
-          <t>Observation Result</t>
-        </is>
-      </c>
-      <c r="P480" s="20" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
+      <c r="M480" s="20" t="inlineStr"/>
+      <c r="N480" s="20" t="n"/>
+      <c r="O480" s="20" t="inlineStr"/>
+      <c r="P480" s="20" t="inlineStr"/>
       <c r="Q480" s="21" t="inlineStr"/>
     </row>
     <row r="481">
@@ -36520,22 +36520,22 @@
       <c r="L481" s="20" t="inlineStr"/>
       <c r="M481" s="20" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="N481" s="22" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="O481" s="20" t="inlineStr">
         <is>
-          <t>Collection Date Time</t>
+          <t>Observation Result</t>
         </is>
       </c>
       <c r="P481" s="20" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="Q481" s="21" t="inlineStr"/>
@@ -36548,17 +36548,17 @@
       </c>
       <c r="B482" s="21" t="inlineStr">
         <is>
-          <t>Pulmonary Reactance</t>
+          <t>Pulmonary Inertance</t>
         </is>
       </c>
       <c r="C482" s="20" t="inlineStr">
         <is>
-          <t>C123567</t>
+          <t>C139254</t>
         </is>
       </c>
       <c r="D482" s="22" t="inlineStr">
         <is>
-          <t>C123567</t>
+          <t>C139254</t>
         </is>
       </c>
       <c r="E482" s="22" t="inlineStr">
@@ -36573,7 +36573,7 @@
       </c>
       <c r="G482" s="20" t="inlineStr">
         <is>
-          <t>PLMXRS</t>
+          <t>INERTANC;Inertance</t>
         </is>
       </c>
       <c r="H482" s="20" t="inlineStr">
@@ -36583,7 +36583,7 @@
       </c>
       <c r="I482" s="21" t="inlineStr">
         <is>
-          <t>The measurement of the ability of the lung to store energy, which is required for passive expiration. Reactance consists of two components: the negative component reflects capacitive behavior (C) and corresponds to both the thoraco-pulmonary elasticity and to changes in the available lung volumes in the distal compartments of the lung; the positive component of reactance has inertial characteristics (I) describing the moving air column in the bronchial tree.</t>
+          <t>The measure of the force of the column of air in the conducting airways.</t>
         </is>
       </c>
       <c r="J482" s="20" t="inlineStr"/>
@@ -36591,22 +36591,22 @@
       <c r="L482" s="20" t="inlineStr"/>
       <c r="M482" s="20" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="N482" s="22" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="O482" s="20" t="inlineStr">
         <is>
-          <t>Observation Result</t>
+          <t>Collection Date Time</t>
         </is>
       </c>
       <c r="P482" s="20" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="Q482" s="21" t="inlineStr"/>
@@ -36662,22 +36662,22 @@
       <c r="L483" s="20" t="inlineStr"/>
       <c r="M483" s="20" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="N483" s="22" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="O483" s="20" t="inlineStr">
         <is>
-          <t>Collection Date Time</t>
+          <t>Observation Result</t>
         </is>
       </c>
       <c r="P483" s="20" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="Q483" s="21" t="inlineStr"/>
@@ -36690,32 +36690,32 @@
       </c>
       <c r="B484" s="21" t="inlineStr">
         <is>
-          <t>Pulse Pressure</t>
+          <t>Pulmonary Reactance</t>
         </is>
       </c>
       <c r="C484" s="20" t="inlineStr">
         <is>
-          <t>C100945</t>
+          <t>C123567</t>
         </is>
       </c>
       <c r="D484" s="22" t="inlineStr">
         <is>
-          <t>C100945</t>
+          <t>C123567</t>
         </is>
       </c>
       <c r="E484" s="22" t="inlineStr">
         <is>
-          <t>C19332</t>
+          <t>C38081</t>
         </is>
       </c>
       <c r="F484" s="21" t="inlineStr">
         <is>
-          <t>Vital Signs;Blood Pressure</t>
+          <t>Respiratory System Findings;Pulmonary Function Test</t>
         </is>
       </c>
       <c r="G484" s="20" t="inlineStr">
         <is>
-          <t>PULSEPR</t>
+          <t>PLMXRS</t>
         </is>
       </c>
       <c r="H484" s="20" t="inlineStr">
@@ -36725,49 +36725,33 @@
       </c>
       <c r="I484" s="21" t="inlineStr">
         <is>
-          <t>The force of a heart contraction measured by the difference between the diastolic and systolic blood pressure measurements.</t>
-        </is>
-      </c>
-      <c r="J484" s="20" t="inlineStr">
-        <is>
-          <t>http://loinc.org/</t>
-        </is>
-      </c>
-      <c r="K484" s="20" t="inlineStr">
-        <is>
-          <t>LOINC</t>
-        </is>
-      </c>
-      <c r="L484" s="20" t="inlineStr">
-        <is>
-          <t>107146-3</t>
-        </is>
-      </c>
+          <t>The measurement of the ability of the lung to store energy, which is required for passive expiration. Reactance consists of two components: the negative component reflects capacitive behavior (C) and corresponds to both the thoraco-pulmonary elasticity and to changes in the available lung volumes in the distal compartments of the lung; the positive component of reactance has inertial characteristics (I) describing the moving air column in the bronchial tree.</t>
+        </is>
+      </c>
+      <c r="J484" s="20" t="inlineStr"/>
+      <c r="K484" s="20" t="inlineStr"/>
+      <c r="L484" s="20" t="inlineStr"/>
       <c r="M484" s="20" t="inlineStr">
         <is>
-          <t>C49669</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="N484" s="22" t="inlineStr">
         <is>
-          <t>C49669</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="O484" s="20" t="inlineStr">
         <is>
-          <t>Unit of Pressure</t>
+          <t>Collection Date Time</t>
         </is>
       </c>
       <c r="P484" s="20" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="Q484" s="21" t="inlineStr">
-        <is>
-          <t>mmHg</t>
-        </is>
-      </c>
+          <t>datetime</t>
+        </is>
+      </c>
+      <c r="Q484" s="21" t="inlineStr"/>
     </row>
     <row r="485">
       <c r="A485" s="20" t="inlineStr">
@@ -36832,25 +36816,29 @@
       </c>
       <c r="M485" s="20" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C49669</t>
         </is>
       </c>
       <c r="N485" s="22" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C49669</t>
         </is>
       </c>
       <c r="O485" s="20" t="inlineStr">
         <is>
-          <t>Observation Result</t>
+          <t>Unit of Pressure</t>
         </is>
       </c>
       <c r="P485" s="20" t="inlineStr">
         <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="Q485" s="21" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="Q485" s="21" t="inlineStr">
+        <is>
+          <t>mmHg</t>
+        </is>
+      </c>
     </row>
     <row r="486">
       <c r="A486" s="20" t="inlineStr">
@@ -37030,32 +37018,32 @@
       </c>
       <c r="B488" s="21" t="inlineStr">
         <is>
-          <t>Quasi-Static Compliance</t>
+          <t>Pulse Pressure</t>
         </is>
       </c>
       <c r="C488" s="20" t="inlineStr">
         <is>
-          <t>C139255</t>
+          <t>C100945</t>
         </is>
       </c>
       <c r="D488" s="22" t="inlineStr">
         <is>
-          <t>C139255</t>
+          <t>C100945</t>
         </is>
       </c>
       <c r="E488" s="22" t="inlineStr">
         <is>
-          <t>C38081</t>
+          <t>C19332</t>
         </is>
       </c>
       <c r="F488" s="21" t="inlineStr">
         <is>
-          <t>Respiratory System Findings;Pulmonary Function Test</t>
+          <t>Vital Signs;Blood Pressure</t>
         </is>
       </c>
       <c r="G488" s="20" t="inlineStr">
         <is>
-          <t>QUASCOMP</t>
+          <t>PULSEPR</t>
         </is>
       </c>
       <c r="H488" s="20" t="inlineStr">
@@ -37065,37 +37053,45 @@
       </c>
       <c r="I488" s="21" t="inlineStr">
         <is>
-          <t>The static elastic recoil pressure of the lungs at a given lung volume.</t>
-        </is>
-      </c>
-      <c r="J488" s="20" t="inlineStr"/>
-      <c r="K488" s="20" t="inlineStr"/>
-      <c r="L488" s="20" t="inlineStr"/>
+          <t>The force of a heart contraction measured by the difference between the diastolic and systolic blood pressure measurements.</t>
+        </is>
+      </c>
+      <c r="J488" s="20" t="inlineStr">
+        <is>
+          <t>http://loinc.org/</t>
+        </is>
+      </c>
+      <c r="K488" s="20" t="inlineStr">
+        <is>
+          <t>LOINC</t>
+        </is>
+      </c>
+      <c r="L488" s="20" t="inlineStr">
+        <is>
+          <t>107146-3</t>
+        </is>
+      </c>
       <c r="M488" s="20" t="inlineStr">
         <is>
-          <t>C49669</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="N488" s="22" t="inlineStr">
         <is>
-          <t>C49669</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="O488" s="20" t="inlineStr">
         <is>
-          <t>Unit of Pressure</t>
+          <t>Observation Result</t>
         </is>
       </c>
       <c r="P488" s="20" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="Q488" s="21" t="inlineStr">
-        <is>
-          <t>mL/cm H2O</t>
-        </is>
-      </c>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="Q488" s="21" t="inlineStr"/>
     </row>
     <row r="489">
       <c r="A489" s="20" t="inlineStr">
@@ -37247,17 +37243,17 @@
       </c>
       <c r="B491" s="21" t="inlineStr">
         <is>
-          <t>Residual Volume</t>
+          <t>Quasi-Static Compliance</t>
         </is>
       </c>
       <c r="C491" s="20" t="inlineStr">
         <is>
-          <t>C89836</t>
+          <t>C139255</t>
         </is>
       </c>
       <c r="D491" s="22" t="inlineStr">
         <is>
-          <t>C89836</t>
+          <t>C139255</t>
         </is>
       </c>
       <c r="E491" s="22" t="inlineStr">
@@ -37272,7 +37268,7 @@
       </c>
       <c r="G491" s="20" t="inlineStr">
         <is>
-          <t>RV</t>
+          <t>QUASCOMP</t>
         </is>
       </c>
       <c r="H491" s="20" t="inlineStr">
@@ -37282,45 +37278,37 @@
       </c>
       <c r="I491" s="21" t="inlineStr">
         <is>
-          <t>The volume of air remaining in the lungs after a maximal exhalation.</t>
-        </is>
-      </c>
-      <c r="J491" s="20" t="inlineStr">
-        <is>
-          <t>http://loinc.org/</t>
-        </is>
-      </c>
-      <c r="K491" s="20" t="inlineStr">
-        <is>
-          <t>LOINC</t>
-        </is>
-      </c>
-      <c r="L491" s="20" t="inlineStr">
-        <is>
-          <t>20146-7</t>
-        </is>
-      </c>
+          <t>The static elastic recoil pressure of the lungs at a given lung volume.</t>
+        </is>
+      </c>
+      <c r="J491" s="20" t="inlineStr"/>
+      <c r="K491" s="20" t="inlineStr"/>
+      <c r="L491" s="20" t="inlineStr"/>
       <c r="M491" s="20" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C49669</t>
         </is>
       </c>
       <c r="N491" s="22" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C49669</t>
         </is>
       </c>
       <c r="O491" s="20" t="inlineStr">
         <is>
-          <t>Collection Date Time</t>
+          <t>Unit of Pressure</t>
         </is>
       </c>
       <c r="P491" s="20" t="inlineStr">
         <is>
-          <t>datetime</t>
-        </is>
-      </c>
-      <c r="Q491" s="21" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="Q491" s="21" t="inlineStr">
+        <is>
+          <t>mL/cm H2O</t>
+        </is>
+      </c>
     </row>
     <row r="492">
       <c r="A492" s="20" t="inlineStr">
@@ -37385,25 +37373,29 @@
       </c>
       <c r="M492" s="20" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C44279</t>
         </is>
       </c>
       <c r="N492" s="22" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C44279</t>
         </is>
       </c>
       <c r="O492" s="20" t="inlineStr">
         <is>
-          <t>Observation Result</t>
+          <t>Unit of Volume</t>
         </is>
       </c>
       <c r="P492" s="20" t="inlineStr">
         <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="Q492" s="21" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="Q492" s="21" t="inlineStr">
+        <is>
+          <t>mL</t>
+        </is>
+      </c>
     </row>
     <row r="493">
       <c r="A493" s="20" t="inlineStr">
@@ -37468,29 +37460,25 @@
       </c>
       <c r="M493" s="20" t="inlineStr">
         <is>
-          <t>C44279</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="N493" s="22" t="inlineStr">
         <is>
-          <t>C44279</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="O493" s="20" t="inlineStr">
         <is>
-          <t>Unit of Volume</t>
+          <t>Collection Date Time</t>
         </is>
       </c>
       <c r="P493" s="20" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="Q493" s="21" t="inlineStr">
-        <is>
-          <t>mL</t>
-        </is>
-      </c>
+          <t>datetime</t>
+        </is>
+      </c>
+      <c r="Q493" s="21" t="inlineStr"/>
     </row>
     <row r="494">
       <c r="A494" s="20" t="inlineStr">
@@ -37500,17 +37488,17 @@
       </c>
       <c r="B494" s="21" t="inlineStr">
         <is>
-          <t>Respiratory Exchange Ratio</t>
+          <t>Residual Volume</t>
         </is>
       </c>
       <c r="C494" s="20" t="inlineStr">
         <is>
-          <t>C123568</t>
+          <t>C89836</t>
         </is>
       </c>
       <c r="D494" s="22" t="inlineStr">
         <is>
-          <t>C123568</t>
+          <t>C89836</t>
         </is>
       </c>
       <c r="E494" s="22" t="inlineStr">
@@ -37525,7 +37513,7 @@
       </c>
       <c r="G494" s="20" t="inlineStr">
         <is>
-          <t>RER</t>
+          <t>RV</t>
         </is>
       </c>
       <c r="H494" s="20" t="inlineStr">
@@ -37535,12 +37523,24 @@
       </c>
       <c r="I494" s="21" t="inlineStr">
         <is>
-          <t>The ratio of the amount of carbon dioxide produced to the amount of oxygen consumed in one breath. This ratio is used to estimate the respiratory quotient, which indicates what type of fuel source the body is metabolising to provide energy.</t>
-        </is>
-      </c>
-      <c r="J494" s="20" t="inlineStr"/>
-      <c r="K494" s="20" t="inlineStr"/>
-      <c r="L494" s="20" t="inlineStr"/>
+          <t>The volume of air remaining in the lungs after a maximal exhalation.</t>
+        </is>
+      </c>
+      <c r="J494" s="20" t="inlineStr">
+        <is>
+          <t>http://loinc.org/</t>
+        </is>
+      </c>
+      <c r="K494" s="20" t="inlineStr">
+        <is>
+          <t>LOINC</t>
+        </is>
+      </c>
+      <c r="L494" s="20" t="inlineStr">
+        <is>
+          <t>20146-7</t>
+        </is>
+      </c>
       <c r="M494" s="20" t="inlineStr">
         <is>
           <t>C70856</t>
@@ -37717,42 +37717,42 @@
       </c>
       <c r="B497" s="21" t="inlineStr">
         <is>
-          <t>Respiratory System Examination</t>
+          <t>Respiratory Exchange Ratio</t>
         </is>
       </c>
       <c r="C497" s="20" t="inlineStr">
         <is>
-          <t>C198356</t>
+          <t>C123568</t>
         </is>
       </c>
       <c r="D497" s="22" t="inlineStr">
         <is>
-          <t>C198356</t>
+          <t>C123568</t>
         </is>
       </c>
       <c r="E497" s="22" t="inlineStr">
         <is>
-          <t>C215116</t>
+          <t>C38081</t>
         </is>
       </c>
       <c r="F497" s="21" t="inlineStr">
         <is>
-          <t>Respiratory System Findings</t>
+          <t>Respiratory System Findings;Pulmonary Function Test</t>
         </is>
       </c>
       <c r="G497" s="20" t="inlineStr">
         <is>
-          <t>REEXAM</t>
+          <t>RER</t>
         </is>
       </c>
       <c r="H497" s="20" t="inlineStr">
         <is>
-          <t>Nominal;Narrative</t>
+          <t>Quantitative</t>
         </is>
       </c>
       <c r="I497" s="21" t="inlineStr">
         <is>
-          <t>An observation, assessment or examination of the respiratory system.</t>
+          <t>The ratio of the amount of carbon dioxide produced to the amount of oxygen consumed in one breath. This ratio is used to estimate the respiratory quotient, which indicates what type of fuel source the body is metabolising to provide energy.</t>
         </is>
       </c>
       <c r="J497" s="20" t="inlineStr"/>
@@ -37760,22 +37760,22 @@
       <c r="L497" s="20" t="inlineStr"/>
       <c r="M497" s="20" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="N497" s="22" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="O497" s="20" t="inlineStr">
         <is>
-          <t>Collection Date Time</t>
+          <t>Observation Result</t>
         </is>
       </c>
       <c r="P497" s="20" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="Q497" s="21" t="inlineStr"/>
@@ -37831,22 +37831,22 @@
       <c r="L498" s="20" t="inlineStr"/>
       <c r="M498" s="20" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="N498" s="22" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="O498" s="20" t="inlineStr">
         <is>
-          <t>Observation Result</t>
+          <t>Collection Date Time</t>
         </is>
       </c>
       <c r="P498" s="20" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="Q498" s="21" t="inlineStr"/>
@@ -37859,20 +37859,24 @@
       </c>
       <c r="B499" s="21" t="inlineStr">
         <is>
-          <t>Respiratory System Finding</t>
+          <t>Respiratory System Examination</t>
         </is>
       </c>
       <c r="C499" s="20" t="inlineStr">
         <is>
-          <t>C45233</t>
+          <t>C198356</t>
         </is>
       </c>
       <c r="D499" s="22" t="inlineStr">
         <is>
-          <t>C45233</t>
-        </is>
-      </c>
-      <c r="E499" s="20" t="n"/>
+          <t>C198356</t>
+        </is>
+      </c>
+      <c r="E499" s="22" t="inlineStr">
+        <is>
+          <t>C215116</t>
+        </is>
+      </c>
       <c r="F499" s="21" t="inlineStr">
         <is>
           <t>Respiratory System Findings</t>
@@ -37880,22 +37884,42 @@
       </c>
       <c r="G499" s="20" t="inlineStr">
         <is>
-          <t>Respiratory;RESPIRATORY SYSTEM;Respiratory Finding</t>
-        </is>
-      </c>
-      <c r="H499" s="20" t="inlineStr"/>
+          <t>REEXAM</t>
+        </is>
+      </c>
+      <c r="H499" s="20" t="inlineStr">
+        <is>
+          <t>Nominal;Narrative</t>
+        </is>
+      </c>
       <c r="I499" s="21" t="inlineStr">
         <is>
-          <t>Symptoms, physical examination results, and/or laboratory test results related to the respiratory system.</t>
+          <t>An observation, assessment or examination of the respiratory system.</t>
         </is>
       </c>
       <c r="J499" s="20" t="inlineStr"/>
       <c r="K499" s="20" t="inlineStr"/>
       <c r="L499" s="20" t="inlineStr"/>
-      <c r="M499" s="20" t="inlineStr"/>
-      <c r="N499" s="20" t="n"/>
-      <c r="O499" s="20" t="inlineStr"/>
-      <c r="P499" s="20" t="inlineStr"/>
+      <c r="M499" s="20" t="inlineStr">
+        <is>
+          <t>C70856</t>
+        </is>
+      </c>
+      <c r="N499" s="22" t="inlineStr">
+        <is>
+          <t>C70856</t>
+        </is>
+      </c>
+      <c r="O499" s="20" t="inlineStr">
+        <is>
+          <t>Observation Result</t>
+        </is>
+      </c>
+      <c r="P499" s="20" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="Q499" s="21" t="inlineStr"/>
     </row>
     <row r="500">
@@ -37906,72 +37930,44 @@
       </c>
       <c r="B500" s="21" t="inlineStr">
         <is>
-          <t>Sagittal Abdominal Diameter</t>
+          <t>Respiratory System Finding</t>
         </is>
       </c>
       <c r="C500" s="20" t="inlineStr">
         <is>
-          <t>C87054</t>
+          <t>C45233</t>
         </is>
       </c>
       <c r="D500" s="22" t="inlineStr">
         <is>
-          <t>C87054</t>
-        </is>
-      </c>
-      <c r="E500" s="22" t="inlineStr">
-        <is>
-          <t>C25285</t>
-        </is>
-      </c>
+          <t>C45233</t>
+        </is>
+      </c>
+      <c r="E500" s="20" t="n"/>
       <c r="F500" s="21" t="inlineStr">
         <is>
-          <t>Vital Signs;Body Measurements</t>
+          <t>Respiratory System Findings</t>
         </is>
       </c>
       <c r="G500" s="20" t="inlineStr">
         <is>
-          <t>SAD</t>
-        </is>
-      </c>
-      <c r="H500" s="20" t="inlineStr">
-        <is>
-          <t>Quantitative</t>
-        </is>
-      </c>
+          <t>Respiratory;RESPIRATORY SYSTEM;Respiratory Finding</t>
+        </is>
+      </c>
+      <c r="H500" s="20" t="inlineStr"/>
       <c r="I500" s="21" t="inlineStr">
         <is>
-          <t>A standard measure of visceral obesity, or abdominal fat, which is measured from the patient's back to upper abdomen between the bottom of the rib cage and the top of the pelvic area. This measurement may be taken with the patient standing or in the supine position.</t>
+          <t>Symptoms, physical examination results, and/or laboratory test results related to the respiratory system.</t>
         </is>
       </c>
       <c r="J500" s="20" t="inlineStr"/>
       <c r="K500" s="20" t="inlineStr"/>
       <c r="L500" s="20" t="inlineStr"/>
-      <c r="M500" s="20" t="inlineStr">
-        <is>
-          <t>C42578</t>
-        </is>
-      </c>
-      <c r="N500" s="22" t="inlineStr">
-        <is>
-          <t>C42578</t>
-        </is>
-      </c>
-      <c r="O500" s="20" t="inlineStr">
-        <is>
-          <t>Unit of Length</t>
-        </is>
-      </c>
-      <c r="P500" s="20" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="Q500" s="21" t="inlineStr">
-        <is>
-          <t>mm;cm;in</t>
-        </is>
-      </c>
+      <c r="M500" s="20" t="inlineStr"/>
+      <c r="N500" s="20" t="n"/>
+      <c r="O500" s="20" t="inlineStr"/>
+      <c r="P500" s="20" t="inlineStr"/>
+      <c r="Q500" s="21" t="inlineStr"/>
     </row>
     <row r="501">
       <c r="A501" s="20" t="inlineStr">
@@ -38095,25 +38091,29 @@
       <c r="L502" s="20" t="inlineStr"/>
       <c r="M502" s="20" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C42578</t>
         </is>
       </c>
       <c r="N502" s="22" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C42578</t>
         </is>
       </c>
       <c r="O502" s="20" t="inlineStr">
         <is>
-          <t>Collection Date Time</t>
+          <t>Unit of Length</t>
         </is>
       </c>
       <c r="P502" s="20" t="inlineStr">
         <is>
-          <t>datetime</t>
-        </is>
-      </c>
-      <c r="Q502" s="21" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="Q502" s="21" t="inlineStr">
+        <is>
+          <t>mm;cm;in</t>
+        </is>
+      </c>
     </row>
     <row r="503">
       <c r="A503" s="20" t="inlineStr">
@@ -38123,32 +38123,32 @@
       </c>
       <c r="B503" s="21" t="inlineStr">
         <is>
-          <t>Salazar-Knowles Equation Parameter A</t>
+          <t>Sagittal Abdominal Diameter</t>
         </is>
       </c>
       <c r="C503" s="20" t="inlineStr">
         <is>
-          <t>C139256</t>
+          <t>C87054</t>
         </is>
       </c>
       <c r="D503" s="22" t="inlineStr">
         <is>
-          <t>C139256</t>
+          <t>C87054</t>
         </is>
       </c>
       <c r="E503" s="22" t="inlineStr">
         <is>
-          <t>C38081</t>
+          <t>C25285</t>
         </is>
       </c>
       <c r="F503" s="21" t="inlineStr">
         <is>
-          <t>Respiratory System Findings;Pulmonary Function Test</t>
+          <t>Vital Signs;Body Measurements</t>
         </is>
       </c>
       <c r="G503" s="20" t="inlineStr">
         <is>
-          <t>SALKA</t>
+          <t>SAD</t>
         </is>
       </c>
       <c r="H503" s="20" t="inlineStr">
@@ -38158,7 +38158,7 @@
       </c>
       <c r="I503" s="21" t="inlineStr">
         <is>
-          <t>A representation of the exponential function described by the Salazar-Knowles equation, and an estimation of a subject's inspiratory capacity.</t>
+          <t>A standard measure of visceral obesity, or abdominal fat, which is measured from the patient's back to upper abdomen between the bottom of the rib cage and the top of the pelvic area. This measurement may be taken with the patient standing or in the supine position.</t>
         </is>
       </c>
       <c r="J503" s="20" t="inlineStr"/>
@@ -38166,22 +38166,22 @@
       <c r="L503" s="20" t="inlineStr"/>
       <c r="M503" s="20" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="N503" s="22" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="O503" s="20" t="inlineStr">
         <is>
-          <t>Observation Result</t>
+          <t>Collection Date Time</t>
         </is>
       </c>
       <c r="P503" s="20" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="Q503" s="21" t="inlineStr"/>
@@ -38265,17 +38265,17 @@
       </c>
       <c r="B505" s="21" t="inlineStr">
         <is>
-          <t>Salazar-Knowles Equation Parameter B</t>
+          <t>Salazar-Knowles Equation Parameter A</t>
         </is>
       </c>
       <c r="C505" s="20" t="inlineStr">
         <is>
-          <t>C139257</t>
+          <t>C139256</t>
         </is>
       </c>
       <c r="D505" s="22" t="inlineStr">
         <is>
-          <t>C139257</t>
+          <t>C139256</t>
         </is>
       </c>
       <c r="E505" s="22" t="inlineStr">
@@ -38290,7 +38290,7 @@
       </c>
       <c r="G505" s="20" t="inlineStr">
         <is>
-          <t>SALKB</t>
+          <t>SALKA</t>
         </is>
       </c>
       <c r="H505" s="20" t="inlineStr">
@@ -38300,7 +38300,7 @@
       </c>
       <c r="I505" s="21" t="inlineStr">
         <is>
-          <t>The difference between the volume at total lung capacity and the hypothesized volume at a transpulmonary pressure of zero.</t>
+          <t>A representation of the exponential function described by the Salazar-Knowles equation, and an estimation of a subject's inspiratory capacity.</t>
         </is>
       </c>
       <c r="J505" s="20" t="inlineStr"/>
@@ -38379,22 +38379,22 @@
       <c r="L506" s="20" t="inlineStr"/>
       <c r="M506" s="20" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="N506" s="22" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="O506" s="20" t="inlineStr">
         <is>
-          <t>Collection Date Time</t>
+          <t>Observation Result</t>
         </is>
       </c>
       <c r="P506" s="20" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="Q506" s="21" t="inlineStr"/>
@@ -38407,17 +38407,17 @@
       </c>
       <c r="B507" s="21" t="inlineStr">
         <is>
-          <t>Salazar-Knowles Equation, K Parameter</t>
+          <t>Salazar-Knowles Equation Parameter B</t>
         </is>
       </c>
       <c r="C507" s="20" t="inlineStr">
         <is>
-          <t>C139258</t>
+          <t>C139257</t>
         </is>
       </c>
       <c r="D507" s="22" t="inlineStr">
         <is>
-          <t>C139258</t>
+          <t>C139257</t>
         </is>
       </c>
       <c r="E507" s="22" t="inlineStr">
@@ -38432,7 +38432,7 @@
       </c>
       <c r="G507" s="20" t="inlineStr">
         <is>
-          <t>Salazar-Knowles Equation, K;SALKK</t>
+          <t>SALKB</t>
         </is>
       </c>
       <c r="H507" s="20" t="inlineStr">
@@ -38442,7 +38442,7 @@
       </c>
       <c r="I507" s="21" t="inlineStr">
         <is>
-          <t>The reflection of the curvature of the upper portion of the deflationary limb of the pressure-volume curve.</t>
+          <t>The difference between the volume at total lung capacity and the hypothesized volume at a transpulmonary pressure of zero.</t>
         </is>
       </c>
       <c r="J507" s="20" t="inlineStr"/>
@@ -38549,32 +38549,32 @@
       </c>
       <c r="B509" s="21" t="inlineStr">
         <is>
-          <t>Second Ventilatory Threshold</t>
+          <t>Salazar-Knowles Equation, K Parameter</t>
         </is>
       </c>
       <c r="C509" s="20" t="inlineStr">
         <is>
-          <t>C204693</t>
+          <t>C139258</t>
         </is>
       </c>
       <c r="D509" s="22" t="inlineStr">
         <is>
-          <t>C204693</t>
+          <t>C139258</t>
         </is>
       </c>
       <c r="E509" s="22" t="inlineStr">
         <is>
-          <t>C123909</t>
+          <t>C38081</t>
         </is>
       </c>
       <c r="F509" s="21" t="inlineStr">
         <is>
-          <t>Respiratory System Findings</t>
+          <t>Respiratory System Findings;Pulmonary Function Test</t>
         </is>
       </c>
       <c r="G509" s="20" t="inlineStr">
         <is>
-          <t>Anaerobic Threshold;Lactate Threshold;Respiratory Compensation Threshold;Ventilatory Threshold 2;VT2</t>
+          <t>Salazar-Knowles Equation, K;SALKK</t>
         </is>
       </c>
       <c r="H509" s="20" t="inlineStr">
@@ -38584,7 +38584,7 @@
       </c>
       <c r="I509" s="21" t="inlineStr">
         <is>
-          <t>The point during activity or exercise at which the effort to ventilate increases such that the exerciser experiences duress and can no longer speak. This threshold is characterized by anaerobic metabolism and lactate buildup.</t>
+          <t>The reflection of the curvature of the upper portion of the deflationary limb of the pressure-volume curve.</t>
         </is>
       </c>
       <c r="J509" s="20" t="inlineStr"/>
@@ -38592,29 +38592,25 @@
       <c r="L509" s="20" t="inlineStr"/>
       <c r="M509" s="20" t="inlineStr">
         <is>
-          <t>C66973</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="N509" s="22" t="inlineStr">
         <is>
-          <t>C66973</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="O509" s="20" t="inlineStr">
         <is>
-          <t>Unit of Dose Calculation</t>
+          <t>Collection Date Time</t>
         </is>
       </c>
       <c r="P509" s="20" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="Q509" s="21" t="inlineStr">
-        <is>
-          <t>mL/kg/min</t>
-        </is>
-      </c>
+          <t>datetime</t>
+        </is>
+      </c>
+      <c r="Q509" s="21" t="inlineStr"/>
     </row>
     <row r="510">
       <c r="A510" s="20" t="inlineStr">
@@ -38667,25 +38663,29 @@
       <c r="L510" s="20" t="inlineStr"/>
       <c r="M510" s="20" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C66973</t>
         </is>
       </c>
       <c r="N510" s="22" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C66973</t>
         </is>
       </c>
       <c r="O510" s="20" t="inlineStr">
         <is>
-          <t>Collection Date Time</t>
+          <t>Unit of Dose Calculation</t>
         </is>
       </c>
       <c r="P510" s="20" t="inlineStr">
         <is>
-          <t>datetime</t>
-        </is>
-      </c>
-      <c r="Q510" s="21" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="Q510" s="21" t="inlineStr">
+        <is>
+          <t>mL/kg/min</t>
+        </is>
+      </c>
     </row>
     <row r="511">
       <c r="A511" s="20" t="inlineStr">
@@ -38766,43 +38766,67 @@
       </c>
       <c r="B512" s="21" t="inlineStr">
         <is>
-          <t>Skinfold Thickness Analysis</t>
+          <t>Second Ventilatory Threshold</t>
         </is>
       </c>
       <c r="C512" s="20" t="inlineStr">
         <is>
-          <t>C77537</t>
+          <t>C204693</t>
         </is>
       </c>
       <c r="D512" s="22" t="inlineStr">
         <is>
-          <t>C77537</t>
-        </is>
-      </c>
-      <c r="E512" s="20" t="n"/>
+          <t>C204693</t>
+        </is>
+      </c>
+      <c r="E512" s="22" t="inlineStr">
+        <is>
+          <t>C123909</t>
+        </is>
+      </c>
       <c r="F512" s="21" t="inlineStr">
         <is>
-          <t>Vital Signs;Body Measurements</t>
+          <t>Respiratory System Findings</t>
         </is>
       </c>
       <c r="G512" s="20" t="inlineStr">
         <is>
-          <t>Skinfold Test</t>
-        </is>
-      </c>
-      <c r="H512" s="20" t="inlineStr"/>
+          <t>Anaerobic Threshold;Lactate Threshold;Respiratory Compensation Threshold;Ventilatory Threshold 2;VT2</t>
+        </is>
+      </c>
+      <c r="H512" s="20" t="inlineStr">
+        <is>
+          <t>Quantitative</t>
+        </is>
+      </c>
       <c r="I512" s="21" t="inlineStr">
         <is>
-          <t>Techniques for estimating body fat whereby a pinch of skin is precisely measured by calipers at several standardized points on the body to determine the subcutaneous fat layer thickness. These measurements are converted to an estimated body fat percentage by an equation.</t>
+          <t>The point during activity or exercise at which the effort to ventilate increases such that the exerciser experiences duress and can no longer speak. This threshold is characterized by anaerobic metabolism and lactate buildup.</t>
         </is>
       </c>
       <c r="J512" s="20" t="inlineStr"/>
       <c r="K512" s="20" t="inlineStr"/>
       <c r="L512" s="20" t="inlineStr"/>
-      <c r="M512" s="20" t="inlineStr"/>
-      <c r="N512" s="20" t="n"/>
-      <c r="O512" s="20" t="inlineStr"/>
-      <c r="P512" s="20" t="inlineStr"/>
+      <c r="M512" s="20" t="inlineStr">
+        <is>
+          <t>C82515</t>
+        </is>
+      </c>
+      <c r="N512" s="22" t="inlineStr">
+        <is>
+          <t>C82515</t>
+        </is>
+      </c>
+      <c r="O512" s="20" t="inlineStr">
+        <is>
+          <t>Collection Date Time</t>
+        </is>
+      </c>
+      <c r="P512" s="20" t="inlineStr">
+        <is>
+          <t>datetime</t>
+        </is>
+      </c>
       <c r="Q512" s="21" t="inlineStr"/>
     </row>
     <row r="513">
@@ -38813,72 +38837,44 @@
       </c>
       <c r="B513" s="21" t="inlineStr">
         <is>
-          <t>Slow Vital Capacity</t>
+          <t>Skinfold Thickness Analysis</t>
         </is>
       </c>
       <c r="C513" s="20" t="inlineStr">
         <is>
-          <t>C111315</t>
+          <t>C77537</t>
         </is>
       </c>
       <c r="D513" s="22" t="inlineStr">
         <is>
-          <t>C111315</t>
-        </is>
-      </c>
-      <c r="E513" s="22" t="inlineStr">
-        <is>
-          <t>C38081</t>
-        </is>
-      </c>
+          <t>C77537</t>
+        </is>
+      </c>
+      <c r="E513" s="20" t="n"/>
       <c r="F513" s="21" t="inlineStr">
         <is>
-          <t>Respiratory System Findings;Pulmonary Function Test</t>
+          <t>Vital Signs;Body Measurements</t>
         </is>
       </c>
       <c r="G513" s="20" t="inlineStr">
         <is>
-          <t>SVC</t>
-        </is>
-      </c>
-      <c r="H513" s="20" t="inlineStr">
-        <is>
-          <t>Quantitative</t>
-        </is>
-      </c>
+          <t>Skinfold Test</t>
+        </is>
+      </c>
+      <c r="H513" s="20" t="inlineStr"/>
       <c r="I513" s="21" t="inlineStr">
         <is>
-          <t>The maximum volume of air that can be exhaled after slow maximum inhalation.</t>
+          <t>Techniques for estimating body fat whereby a pinch of skin is precisely measured by calipers at several standardized points on the body to determine the subcutaneous fat layer thickness. These measurements are converted to an estimated body fat percentage by an equation.</t>
         </is>
       </c>
       <c r="J513" s="20" t="inlineStr"/>
       <c r="K513" s="20" t="inlineStr"/>
       <c r="L513" s="20" t="inlineStr"/>
-      <c r="M513" s="20" t="inlineStr">
-        <is>
-          <t>C44279</t>
-        </is>
-      </c>
-      <c r="N513" s="22" t="inlineStr">
-        <is>
-          <t>C44279</t>
-        </is>
-      </c>
-      <c r="O513" s="20" t="inlineStr">
-        <is>
-          <t>Unit of Volume</t>
-        </is>
-      </c>
-      <c r="P513" s="20" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="Q513" s="21" t="inlineStr">
-        <is>
-          <t>L;mL</t>
-        </is>
-      </c>
+      <c r="M513" s="20" t="inlineStr"/>
+      <c r="N513" s="20" t="n"/>
+      <c r="O513" s="20" t="inlineStr"/>
+      <c r="P513" s="20" t="inlineStr"/>
+      <c r="Q513" s="21" t="inlineStr"/>
     </row>
     <row r="514">
       <c r="A514" s="20" t="inlineStr">
@@ -39002,25 +38998,29 @@
       <c r="L515" s="20" t="inlineStr"/>
       <c r="M515" s="20" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C44279</t>
         </is>
       </c>
       <c r="N515" s="22" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C44279</t>
         </is>
       </c>
       <c r="O515" s="20" t="inlineStr">
         <is>
-          <t>Observation Result</t>
+          <t>Unit of Volume</t>
         </is>
       </c>
       <c r="P515" s="20" t="inlineStr">
         <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="Q515" s="21" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="Q515" s="21" t="inlineStr">
+        <is>
+          <t>L;mL</t>
+        </is>
+      </c>
     </row>
     <row r="516">
       <c r="A516" s="20" t="inlineStr">
@@ -39030,17 +39030,17 @@
       </c>
       <c r="B516" s="21" t="inlineStr">
         <is>
-          <t>Specific Airway Conductance</t>
+          <t>Slow Vital Capacity</t>
         </is>
       </c>
       <c r="C516" s="20" t="inlineStr">
         <is>
-          <t>C122186</t>
+          <t>C111315</t>
         </is>
       </c>
       <c r="D516" s="22" t="inlineStr">
         <is>
-          <t>C122186</t>
+          <t>C111315</t>
         </is>
       </c>
       <c r="E516" s="22" t="inlineStr">
@@ -39055,7 +39055,7 @@
       </c>
       <c r="G516" s="20" t="inlineStr">
         <is>
-          <t>SGAW;sGaw</t>
+          <t>SVC</t>
         </is>
       </c>
       <c r="H516" s="20" t="inlineStr">
@@ -39065,7 +39065,7 @@
       </c>
       <c r="I516" s="21" t="inlineStr">
         <is>
-          <t>A measurement of the airway conductance relative to lung volume.</t>
+          <t>The maximum volume of air that can be exhaled after slow maximum inhalation.</t>
         </is>
       </c>
       <c r="J516" s="20" t="inlineStr"/>
@@ -39073,22 +39073,22 @@
       <c r="L516" s="20" t="inlineStr"/>
       <c r="M516" s="20" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="N516" s="22" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="O516" s="20" t="inlineStr">
         <is>
-          <t>Collection Date Time</t>
+          <t>Observation Result</t>
         </is>
       </c>
       <c r="P516" s="20" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="Q516" s="21" t="inlineStr"/>
@@ -39172,17 +39172,17 @@
       </c>
       <c r="B518" s="21" t="inlineStr">
         <is>
-          <t>Specific Airway Resistance</t>
+          <t>Specific Airway Conductance</t>
         </is>
       </c>
       <c r="C518" s="20" t="inlineStr">
         <is>
-          <t>C123569</t>
+          <t>C122186</t>
         </is>
       </c>
       <c r="D518" s="22" t="inlineStr">
         <is>
-          <t>C123569</t>
+          <t>C122186</t>
         </is>
       </c>
       <c r="E518" s="22" t="inlineStr">
@@ -39197,7 +39197,7 @@
       </c>
       <c r="G518" s="20" t="inlineStr">
         <is>
-          <t>SRAW;sRAW</t>
+          <t>SGAW;sGaw</t>
         </is>
       </c>
       <c r="H518" s="20" t="inlineStr">
@@ -39207,7 +39207,7 @@
       </c>
       <c r="I518" s="21" t="inlineStr">
         <is>
-          <t>A measurement used to describe airway behavior irrespective of lung volume; it is calculated as airway resistance (Raw) multiplied by functional residual capacity (FRC).</t>
+          <t>A measurement of the airway conductance relative to lung volume.</t>
         </is>
       </c>
       <c r="J518" s="20" t="inlineStr"/>
@@ -39215,22 +39215,22 @@
       <c r="L518" s="20" t="inlineStr"/>
       <c r="M518" s="20" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="N518" s="22" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="O518" s="20" t="inlineStr">
         <is>
-          <t>Observation Result</t>
+          <t>Collection Date Time</t>
         </is>
       </c>
       <c r="P518" s="20" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="Q518" s="21" t="inlineStr"/>
@@ -39286,29 +39286,25 @@
       <c r="L519" s="20" t="inlineStr"/>
       <c r="M519" s="20" t="inlineStr">
         <is>
-          <t>C67332</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="N519" s="22" t="inlineStr">
         <is>
-          <t>C67332</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="O519" s="20" t="inlineStr">
         <is>
-          <t>Manometric Unit of Pressure</t>
+          <t>Observation Result</t>
         </is>
       </c>
       <c r="P519" s="20" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="Q519" s="21" t="inlineStr">
-        <is>
-          <t>cmH2O*s/mL</t>
-        </is>
-      </c>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="Q519" s="21" t="inlineStr"/>
     </row>
     <row r="520">
       <c r="A520" s="20" t="inlineStr">
@@ -39361,25 +39357,29 @@
       <c r="L520" s="20" t="inlineStr"/>
       <c r="M520" s="20" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C67332</t>
         </is>
       </c>
       <c r="N520" s="22" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C67332</t>
         </is>
       </c>
       <c r="O520" s="20" t="inlineStr">
         <is>
-          <t>Collection Date Time</t>
+          <t>Manometric Unit of Pressure</t>
         </is>
       </c>
       <c r="P520" s="20" t="inlineStr">
         <is>
-          <t>datetime</t>
-        </is>
-      </c>
-      <c r="Q520" s="21" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="Q520" s="21" t="inlineStr">
+        <is>
+          <t>cmH2O*s/mL</t>
+        </is>
+      </c>
     </row>
     <row r="521">
       <c r="A521" s="20" t="inlineStr">
@@ -39389,32 +39389,32 @@
       </c>
       <c r="B521" s="21" t="inlineStr">
         <is>
-          <t>Specific Airway Volume</t>
+          <t>Specific Airway Resistance</t>
         </is>
       </c>
       <c r="C521" s="20" t="inlineStr">
         <is>
-          <t>C170618</t>
+          <t>C123569</t>
         </is>
       </c>
       <c r="D521" s="22" t="inlineStr">
         <is>
-          <t>C170618</t>
+          <t>C123569</t>
         </is>
       </c>
       <c r="E521" s="22" t="inlineStr">
         <is>
-          <t>C170457</t>
+          <t>C38081</t>
         </is>
       </c>
       <c r="F521" s="21" t="inlineStr">
         <is>
-          <t>Respiratory System Findings</t>
+          <t>Respiratory System Findings;Pulmonary Function Test</t>
         </is>
       </c>
       <c r="G521" s="20" t="inlineStr">
         <is>
-          <t>SAWVOL</t>
+          <t>SRAW;sRAW</t>
         </is>
       </c>
       <c r="H521" s="20" t="inlineStr">
@@ -39424,7 +39424,7 @@
       </c>
       <c r="I521" s="21" t="inlineStr">
         <is>
-          <t>A parameter used in functional respiratory imaging, derived by dividing the airway volume of a specified intrapulmonary region by the total volume of the same specified intrapulmonary region.</t>
+          <t>A measurement used to describe airway behavior irrespective of lung volume; it is calculated as airway resistance (Raw) multiplied by functional residual capacity (FRC).</t>
         </is>
       </c>
       <c r="J521" s="20" t="inlineStr"/>
@@ -39503,22 +39503,22 @@
       <c r="L522" s="20" t="inlineStr"/>
       <c r="M522" s="20" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="N522" s="22" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="O522" s="20" t="inlineStr">
         <is>
-          <t>Observation Result</t>
+          <t>Collection Date Time</t>
         </is>
       </c>
       <c r="P522" s="20" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="Q522" s="21" t="inlineStr"/>
@@ -39574,29 +39574,25 @@
       <c r="L523" s="20" t="inlineStr"/>
       <c r="M523" s="20" t="inlineStr">
         <is>
-          <t>C44279</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="N523" s="22" t="inlineStr">
         <is>
-          <t>C44279</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="O523" s="20" t="inlineStr">
         <is>
-          <t>Unit of Volume</t>
+          <t>Observation Result</t>
         </is>
       </c>
       <c r="P523" s="20" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="Q523" s="21" t="inlineStr">
-        <is>
-          <t>mL</t>
-        </is>
-      </c>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="Q523" s="21" t="inlineStr"/>
     </row>
     <row r="524">
       <c r="A524" s="20" t="inlineStr">
@@ -39606,32 +39602,32 @@
       </c>
       <c r="B524" s="21" t="inlineStr">
         <is>
-          <t>Subscapular Skinfold Thickness</t>
+          <t>Specific Airway Volume</t>
         </is>
       </c>
       <c r="C524" s="20" t="inlineStr">
         <is>
-          <t>C98785</t>
+          <t>C170618</t>
         </is>
       </c>
       <c r="D524" s="22" t="inlineStr">
         <is>
-          <t>C98785</t>
+          <t>C170618</t>
         </is>
       </c>
       <c r="E524" s="22" t="inlineStr">
         <is>
-          <t>C77537</t>
+          <t>C170457</t>
         </is>
       </c>
       <c r="F524" s="21" t="inlineStr">
         <is>
-          <t>Vital Signs;Body Measurements</t>
+          <t>Respiratory System Findings</t>
         </is>
       </c>
       <c r="G524" s="20" t="inlineStr">
         <is>
-          <t>SSSKNF</t>
+          <t>SAWVOL</t>
         </is>
       </c>
       <c r="H524" s="20" t="inlineStr">
@@ -39641,7 +39637,7 @@
       </c>
       <c r="I524" s="21" t="inlineStr">
         <is>
-          <t>A measurement of the thickness of a pinch of skin situated below or on the underside of the scapula.</t>
+          <t>A parameter used in functional respiratory imaging, derived by dividing the airway volume of a specified intrapulmonary region by the total volume of the same specified intrapulmonary region.</t>
         </is>
       </c>
       <c r="J524" s="20" t="inlineStr"/>
@@ -39649,17 +39645,17 @@
       <c r="L524" s="20" t="inlineStr"/>
       <c r="M524" s="20" t="inlineStr">
         <is>
-          <t>C42578</t>
+          <t>C44279</t>
         </is>
       </c>
       <c r="N524" s="22" t="inlineStr">
         <is>
-          <t>C42578</t>
+          <t>C44279</t>
         </is>
       </c>
       <c r="O524" s="20" t="inlineStr">
         <is>
-          <t>Unit of Length</t>
+          <t>Unit of Volume</t>
         </is>
       </c>
       <c r="P524" s="20" t="inlineStr">
@@ -39669,7 +39665,7 @@
       </c>
       <c r="Q524" s="21" t="inlineStr">
         <is>
-          <t>mm;cm;in</t>
+          <t>mL</t>
         </is>
       </c>
     </row>
@@ -39823,44 +39819,72 @@
       </c>
       <c r="B527" s="21" t="inlineStr">
         <is>
-          <t>Symptom Indicator</t>
+          <t>Subscapular Skinfold Thickness</t>
         </is>
       </c>
       <c r="C527" s="20" t="inlineStr">
         <is>
-          <t>C119241</t>
+          <t>C98785</t>
         </is>
       </c>
       <c r="D527" s="22" t="inlineStr">
         <is>
-          <t>C119241</t>
-        </is>
-      </c>
-      <c r="E527" s="20" t="n"/>
+          <t>C98785</t>
+        </is>
+      </c>
+      <c r="E527" s="22" t="inlineStr">
+        <is>
+          <t>C77537</t>
+        </is>
+      </c>
       <c r="F527" s="21" t="inlineStr">
         <is>
-          <t>Musculoskeletal Finding;Symptom Indicator;Reproductive Findings;Clinical Findings Indicator;Symptom Indicator;Skin Response;Reproductive Findings;Respiratory System Findings</t>
+          <t>Vital Signs;Body Measurements</t>
         </is>
       </c>
       <c r="G527" s="20" t="inlineStr">
         <is>
-          <t>SYMPINDC</t>
-        </is>
-      </c>
-      <c r="H527" s="20" t="inlineStr"/>
+          <t>SSSKNF</t>
+        </is>
+      </c>
+      <c r="H527" s="20" t="inlineStr">
+        <is>
+          <t>Quantitative</t>
+        </is>
+      </c>
       <c r="I527" s="21" t="inlineStr">
         <is>
-          <t>An indication as to whether the subject had symptoms related to the clinical event of interest.</t>
+          <t>A measurement of the thickness of a pinch of skin situated below or on the underside of the scapula.</t>
         </is>
       </c>
       <c r="J527" s="20" t="inlineStr"/>
       <c r="K527" s="20" t="inlineStr"/>
       <c r="L527" s="20" t="inlineStr"/>
-      <c r="M527" s="20" t="inlineStr"/>
-      <c r="N527" s="20" t="n"/>
-      <c r="O527" s="20" t="inlineStr"/>
-      <c r="P527" s="20" t="inlineStr"/>
-      <c r="Q527" s="21" t="inlineStr"/>
+      <c r="M527" s="20" t="inlineStr">
+        <is>
+          <t>C42578</t>
+        </is>
+      </c>
+      <c r="N527" s="22" t="inlineStr">
+        <is>
+          <t>C42578</t>
+        </is>
+      </c>
+      <c r="O527" s="20" t="inlineStr">
+        <is>
+          <t>Unit of Length</t>
+        </is>
+      </c>
+      <c r="P527" s="20" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="Q527" s="21" t="inlineStr">
+        <is>
+          <t>mm;cm;in</t>
+        </is>
+      </c>
     </row>
     <row r="528">
       <c r="A528" s="20" t="inlineStr">
@@ -39870,63 +39894,43 @@
       </c>
       <c r="B528" s="21" t="inlineStr">
         <is>
-          <t>Systolic Blood Pressure-for-Age Percentile</t>
+          <t>Symptom Indicator</t>
         </is>
       </c>
       <c r="C528" s="20" t="inlineStr">
         <is>
-          <t>C172608</t>
+          <t>C119241</t>
         </is>
       </c>
       <c r="D528" s="22" t="inlineStr">
         <is>
-          <t>C172608</t>
+          <t>C119241</t>
         </is>
       </c>
       <c r="E528" s="20" t="n"/>
       <c r="F528" s="21" t="inlineStr">
         <is>
-          <t>Vital Signs;Blood Pressure</t>
+          <t>Musculoskeletal Finding;Symptom Indicator;Reproductive Findings;Clinical Findings Indicator;Symptom Indicator;Skin Response;Reproductive Findings;Respiratory System Findings</t>
         </is>
       </c>
       <c r="G528" s="20" t="inlineStr">
         <is>
-          <t>SBPAPCTL;Systolic BP-for-Age Percentile</t>
-        </is>
-      </c>
-      <c r="H528" s="20" t="inlineStr">
-        <is>
-          <t>Quantitative</t>
-        </is>
-      </c>
+          <t>SYMPINDC</t>
+        </is>
+      </c>
+      <c r="H528" s="20" t="inlineStr"/>
       <c r="I528" s="21" t="inlineStr">
         <is>
-          <t>A measurement of an individual's systolic blood pressure in relationship to age, in comparison to a reference percentile curve.</t>
+          <t>An indication as to whether the subject had symptoms related to the clinical event of interest.</t>
         </is>
       </c>
       <c r="J528" s="20" t="inlineStr"/>
       <c r="K528" s="20" t="inlineStr"/>
       <c r="L528" s="20" t="inlineStr"/>
-      <c r="M528" s="20" t="inlineStr">
-        <is>
-          <t>C82515</t>
-        </is>
-      </c>
-      <c r="N528" s="22" t="inlineStr">
-        <is>
-          <t>C82515</t>
-        </is>
-      </c>
-      <c r="O528" s="20" t="inlineStr">
-        <is>
-          <t>Collection Date Time</t>
-        </is>
-      </c>
-      <c r="P528" s="20" t="inlineStr">
-        <is>
-          <t>datetime</t>
-        </is>
-      </c>
+      <c r="M528" s="20" t="inlineStr"/>
+      <c r="N528" s="20" t="n"/>
+      <c r="O528" s="20" t="inlineStr"/>
+      <c r="P528" s="20" t="inlineStr"/>
       <c r="Q528" s="21" t="inlineStr"/>
     </row>
     <row r="529">
@@ -40004,17 +40008,17 @@
       </c>
       <c r="B530" s="21" t="inlineStr">
         <is>
-          <t>Systolic Blood Pressure-for-Height Percentile</t>
+          <t>Systolic Blood Pressure-for-Age Percentile</t>
         </is>
       </c>
       <c r="C530" s="20" t="inlineStr">
         <is>
-          <t>C172607</t>
+          <t>C172608</t>
         </is>
       </c>
       <c r="D530" s="22" t="inlineStr">
         <is>
-          <t>C172607</t>
+          <t>C172608</t>
         </is>
       </c>
       <c r="E530" s="20" t="n"/>
@@ -40025,7 +40029,7 @@
       </c>
       <c r="G530" s="20" t="inlineStr">
         <is>
-          <t>SBPHPCTL;Systolic BP-for-Height Percentile</t>
+          <t>SBPAPCTL;Systolic BP-for-Age Percentile</t>
         </is>
       </c>
       <c r="H530" s="20" t="inlineStr">
@@ -40035,7 +40039,7 @@
       </c>
       <c r="I530" s="21" t="inlineStr">
         <is>
-          <t>A measurement of an individual's systolic blood pressure in relationship to height, in comparison to a reference percentile curve.</t>
+          <t>A measurement of an individual's systolic blood pressure in relationship to age, in comparison to a reference percentile curve.</t>
         </is>
       </c>
       <c r="J530" s="20" t="inlineStr"/>
@@ -40110,22 +40114,22 @@
       <c r="L531" s="20" t="inlineStr"/>
       <c r="M531" s="20" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="N531" s="22" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="O531" s="20" t="inlineStr">
         <is>
-          <t>Observation Result</t>
+          <t>Collection Date Time</t>
         </is>
       </c>
       <c r="P531" s="20" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="Q531" s="21" t="inlineStr"/>
@@ -40138,32 +40142,28 @@
       </c>
       <c r="B532" s="21" t="inlineStr">
         <is>
-          <t>Thoracic Gas Volume</t>
+          <t>Systolic Blood Pressure-for-Height Percentile</t>
         </is>
       </c>
       <c r="C532" s="20" t="inlineStr">
         <is>
-          <t>C124426</t>
+          <t>C172607</t>
         </is>
       </c>
       <c r="D532" s="22" t="inlineStr">
         <is>
-          <t>C124426</t>
-        </is>
-      </c>
-      <c r="E532" s="22" t="inlineStr">
-        <is>
-          <t>C38081</t>
-        </is>
-      </c>
+          <t>C172607</t>
+        </is>
+      </c>
+      <c r="E532" s="20" t="n"/>
       <c r="F532" s="21" t="inlineStr">
         <is>
-          <t>Respiratory System Findings;Pulmonary Function Test</t>
+          <t>Vital Signs;Blood Pressure</t>
         </is>
       </c>
       <c r="G532" s="20" t="inlineStr">
         <is>
-          <t>TGV</t>
+          <t>SBPHPCTL;Systolic BP-for-Height Percentile</t>
         </is>
       </c>
       <c r="H532" s="20" t="inlineStr">
@@ -40173,42 +40173,30 @@
       </c>
       <c r="I532" s="21" t="inlineStr">
         <is>
-          <t>The absolute volume of gas contained in the thoracic cavity at any given point in time and at any level of alveolar pressure.</t>
-        </is>
-      </c>
-      <c r="J532" s="20" t="inlineStr">
-        <is>
-          <t>http://loinc.org/</t>
-        </is>
-      </c>
-      <c r="K532" s="20" t="inlineStr">
-        <is>
-          <t>LOINC</t>
-        </is>
-      </c>
-      <c r="L532" s="20" t="inlineStr">
-        <is>
-          <t>20132-7</t>
-        </is>
-      </c>
+          <t>A measurement of an individual's systolic blood pressure in relationship to height, in comparison to a reference percentile curve.</t>
+        </is>
+      </c>
+      <c r="J532" s="20" t="inlineStr"/>
+      <c r="K532" s="20" t="inlineStr"/>
+      <c r="L532" s="20" t="inlineStr"/>
       <c r="M532" s="20" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="N532" s="22" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="O532" s="20" t="inlineStr">
         <is>
-          <t>Collection Date Time</t>
+          <t>Observation Result</t>
         </is>
       </c>
       <c r="P532" s="20" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="Q532" s="21" t="inlineStr"/>
@@ -40276,25 +40264,29 @@
       </c>
       <c r="M533" s="20" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C44279</t>
         </is>
       </c>
       <c r="N533" s="22" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C44279</t>
         </is>
       </c>
       <c r="O533" s="20" t="inlineStr">
         <is>
-          <t>Observation Result</t>
+          <t>Unit of Volume</t>
         </is>
       </c>
       <c r="P533" s="20" t="inlineStr">
         <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="Q533" s="21" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="Q533" s="21" t="inlineStr">
+        <is>
+          <t>mL;L</t>
+        </is>
+      </c>
     </row>
     <row r="534">
       <c r="A534" s="20" t="inlineStr">
@@ -40359,29 +40351,25 @@
       </c>
       <c r="M534" s="20" t="inlineStr">
         <is>
-          <t>C44279</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="N534" s="22" t="inlineStr">
         <is>
-          <t>C44279</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="O534" s="20" t="inlineStr">
         <is>
-          <t>Unit of Volume</t>
+          <t>Observation Result</t>
         </is>
       </c>
       <c r="P534" s="20" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="Q534" s="21" t="inlineStr">
-        <is>
-          <t>mL;L</t>
-        </is>
-      </c>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="Q534" s="21" t="inlineStr"/>
     </row>
     <row r="535">
       <c r="A535" s="20" t="inlineStr">
@@ -40391,32 +40379,32 @@
       </c>
       <c r="B535" s="21" t="inlineStr">
         <is>
-          <t>Tibial Length</t>
+          <t>Thoracic Gas Volume</t>
         </is>
       </c>
       <c r="C535" s="20" t="inlineStr">
         <is>
-          <t>C191365</t>
+          <t>C124426</t>
         </is>
       </c>
       <c r="D535" s="22" t="inlineStr">
         <is>
-          <t>C191365</t>
+          <t>C124426</t>
         </is>
       </c>
       <c r="E535" s="22" t="inlineStr">
         <is>
-          <t>C25334</t>
+          <t>C38081</t>
         </is>
       </c>
       <c r="F535" s="21" t="inlineStr">
         <is>
-          <t>Vital Signs;Body Measurements</t>
+          <t>Respiratory System Findings;Pulmonary Function Test</t>
         </is>
       </c>
       <c r="G535" s="20" t="inlineStr">
         <is>
-          <t>TIBIAL</t>
+          <t>TGV</t>
         </is>
       </c>
       <c r="H535" s="20" t="inlineStr">
@@ -40426,30 +40414,42 @@
       </c>
       <c r="I535" s="21" t="inlineStr">
         <is>
-          <t>A measurement of the length of the tibia.</t>
-        </is>
-      </c>
-      <c r="J535" s="20" t="inlineStr"/>
-      <c r="K535" s="20" t="inlineStr"/>
-      <c r="L535" s="20" t="inlineStr"/>
+          <t>The absolute volume of gas contained in the thoracic cavity at any given point in time and at any level of alveolar pressure.</t>
+        </is>
+      </c>
+      <c r="J535" s="20" t="inlineStr">
+        <is>
+          <t>http://loinc.org/</t>
+        </is>
+      </c>
+      <c r="K535" s="20" t="inlineStr">
+        <is>
+          <t>LOINC</t>
+        </is>
+      </c>
+      <c r="L535" s="20" t="inlineStr">
+        <is>
+          <t>20132-7</t>
+        </is>
+      </c>
       <c r="M535" s="20" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="N535" s="22" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="O535" s="20" t="inlineStr">
         <is>
-          <t>Observation Result</t>
+          <t>Collection Date Time</t>
         </is>
       </c>
       <c r="P535" s="20" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="Q535" s="21" t="inlineStr"/>
@@ -40608,32 +40608,32 @@
       </c>
       <c r="B538" s="21" t="inlineStr">
         <is>
-          <t>Tidal Volume</t>
+          <t>Tibial Length</t>
         </is>
       </c>
       <c r="C538" s="20" t="inlineStr">
         <is>
-          <t>C111324</t>
+          <t>C191365</t>
         </is>
       </c>
       <c r="D538" s="22" t="inlineStr">
         <is>
-          <t>C111324</t>
+          <t>C191365</t>
         </is>
       </c>
       <c r="E538" s="22" t="inlineStr">
         <is>
-          <t>C38081</t>
+          <t>C25334</t>
         </is>
       </c>
       <c r="F538" s="21" t="inlineStr">
         <is>
-          <t>Respiratory System Findings;Pulmonary Function Test</t>
+          <t>Vital Signs;Body Measurements</t>
         </is>
       </c>
       <c r="G538" s="20" t="inlineStr">
         <is>
-          <t>TIDALVOL;TV</t>
+          <t>TIBIAL</t>
         </is>
       </c>
       <c r="H538" s="20" t="inlineStr">
@@ -40643,7 +40643,7 @@
       </c>
       <c r="I538" s="21" t="inlineStr">
         <is>
-          <t>The volume of air moved into and out of the lungs during breathing at rest.</t>
+          <t>A measurement of the length of the tibia.</t>
         </is>
       </c>
       <c r="J538" s="20" t="inlineStr"/>
@@ -40722,25 +40722,29 @@
       <c r="L539" s="20" t="inlineStr"/>
       <c r="M539" s="20" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C44279</t>
         </is>
       </c>
       <c r="N539" s="22" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C44279</t>
         </is>
       </c>
       <c r="O539" s="20" t="inlineStr">
         <is>
-          <t>Collection Date Time</t>
+          <t>Unit of Volume</t>
         </is>
       </c>
       <c r="P539" s="20" t="inlineStr">
         <is>
-          <t>datetime</t>
-        </is>
-      </c>
-      <c r="Q539" s="21" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="Q539" s="21" t="inlineStr">
+        <is>
+          <t>mL;L</t>
+        </is>
+      </c>
     </row>
     <row r="540">
       <c r="A540" s="20" t="inlineStr">
@@ -40793,29 +40797,25 @@
       <c r="L540" s="20" t="inlineStr"/>
       <c r="M540" s="20" t="inlineStr">
         <is>
-          <t>C44279</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="N540" s="22" t="inlineStr">
         <is>
-          <t>C44279</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="O540" s="20" t="inlineStr">
         <is>
-          <t>Unit of Volume</t>
+          <t>Collection Date Time</t>
         </is>
       </c>
       <c r="P540" s="20" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="Q540" s="21" t="inlineStr">
-        <is>
-          <t>mL;L</t>
-        </is>
-      </c>
+          <t>datetime</t>
+        </is>
+      </c>
+      <c r="Q540" s="21" t="inlineStr"/>
     </row>
     <row r="541">
       <c r="A541" s="20" t="inlineStr">
@@ -40825,17 +40825,17 @@
       </c>
       <c r="B541" s="21" t="inlineStr">
         <is>
-          <t>Tissue Elastance</t>
+          <t>Tidal Volume</t>
         </is>
       </c>
       <c r="C541" s="20" t="inlineStr">
         <is>
-          <t>C139260</t>
+          <t>C111324</t>
         </is>
       </c>
       <c r="D541" s="22" t="inlineStr">
         <is>
-          <t>C139260</t>
+          <t>C111324</t>
         </is>
       </c>
       <c r="E541" s="22" t="inlineStr">
@@ -40850,7 +40850,7 @@
       </c>
       <c r="G541" s="20" t="inlineStr">
         <is>
-          <t>TSUELAS</t>
+          <t>TIDALVOL;TV</t>
         </is>
       </c>
       <c r="H541" s="20" t="inlineStr">
@@ -40860,7 +40860,7 @@
       </c>
       <c r="I541" s="21" t="inlineStr">
         <is>
-          <t>A reflection of energy conservation within a given tissue.</t>
+          <t>The volume of air moved into and out of the lungs during breathing at rest.</t>
         </is>
       </c>
       <c r="J541" s="20" t="inlineStr"/>
@@ -40868,22 +40868,22 @@
       <c r="L541" s="20" t="inlineStr"/>
       <c r="M541" s="20" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="N541" s="22" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="O541" s="20" t="inlineStr">
         <is>
-          <t>Collection Date Time</t>
+          <t>Observation Result</t>
         </is>
       </c>
       <c r="P541" s="20" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="Q541" s="21" t="inlineStr"/>
@@ -41042,17 +41042,17 @@
       </c>
       <c r="B544" s="21" t="inlineStr">
         <is>
-          <t>Tissue Hysteresivity Measurement</t>
+          <t>Tissue Elastance</t>
         </is>
       </c>
       <c r="C544" s="20" t="inlineStr">
         <is>
-          <t>C139261</t>
+          <t>C139260</t>
         </is>
       </c>
       <c r="D544" s="22" t="inlineStr">
         <is>
-          <t>C139261</t>
+          <t>C139260</t>
         </is>
       </c>
       <c r="E544" s="22" t="inlineStr">
@@ -41067,7 +41067,7 @@
       </c>
       <c r="G544" s="20" t="inlineStr">
         <is>
-          <t>Tissue Hysteresivity;TSUHYS</t>
+          <t>TSUELAS</t>
         </is>
       </c>
       <c r="H544" s="20" t="inlineStr">
@@ -41077,7 +41077,7 @@
       </c>
       <c r="I544" s="21" t="inlineStr">
         <is>
-          <t>The energy dissipated relative to the elastic energy stored in the tissue in a P-V cycle. Fredberg, J.J., Stamenovic, D. (1 December 1989). On the Imperfect Elasticity of Lung Tissue. Journal of Applied Physiology, Vol. 67. Retrieved from https://owl.english.purdue.edu/owl/resource/560/10/</t>
+          <t>A reflection of energy conservation within a given tissue.</t>
         </is>
       </c>
       <c r="J544" s="20" t="inlineStr"/>
@@ -41184,32 +41184,32 @@
       </c>
       <c r="B546" s="21" t="inlineStr">
         <is>
-          <t>Total Body Length</t>
+          <t>Tissue Hysteresivity Measurement</t>
         </is>
       </c>
       <c r="C546" s="20" t="inlineStr">
         <is>
-          <t>C81298</t>
+          <t>C139261</t>
         </is>
       </c>
       <c r="D546" s="22" t="inlineStr">
         <is>
-          <t>C81298</t>
+          <t>C139261</t>
         </is>
       </c>
       <c r="E546" s="22" t="inlineStr">
         <is>
-          <t>C25334</t>
+          <t>C38081</t>
         </is>
       </c>
       <c r="F546" s="21" t="inlineStr">
         <is>
-          <t>Vital Signs;Body Measurements</t>
+          <t>Respiratory System Findings;Pulmonary Function Test</t>
         </is>
       </c>
       <c r="G546" s="20" t="inlineStr">
         <is>
-          <t>BODLNGTH;Body Length</t>
+          <t>Tissue Hysteresivity;TSUHYS</t>
         </is>
       </c>
       <c r="H546" s="20" t="inlineStr">
@@ -41219,7 +41219,7 @@
       </c>
       <c r="I546" s="21" t="inlineStr">
         <is>
-          <t>The total linear extent of the body.</t>
+          <t>The energy dissipated relative to the elastic energy stored in the tissue in a P-V cycle. Fredberg, J.J., Stamenovic, D. (1 December 1989). On the Imperfect Elasticity of Lung Tissue. Journal of Applied Physiology, Vol. 67. Retrieved from https://owl.english.purdue.edu/owl/resource/560/10/</t>
         </is>
       </c>
       <c r="J546" s="20" t="inlineStr"/>
@@ -41373,22 +41373,22 @@
       <c r="L548" s="20" t="inlineStr"/>
       <c r="M548" s="20" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="N548" s="22" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="O548" s="20" t="inlineStr">
         <is>
-          <t>Observation Result</t>
+          <t>Collection Date Time</t>
         </is>
       </c>
       <c r="P548" s="20" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="Q548" s="21" t="inlineStr"/>
@@ -41401,32 +41401,32 @@
       </c>
       <c r="B549" s="21" t="inlineStr">
         <is>
-          <t>Total Body Water Measurement</t>
+          <t>Total Body Length</t>
         </is>
       </c>
       <c r="C549" s="20" t="inlineStr">
         <is>
-          <t>C104622</t>
+          <t>C81298</t>
         </is>
       </c>
       <c r="D549" s="22" t="inlineStr">
         <is>
-          <t>C104622</t>
+          <t>C81298</t>
         </is>
       </c>
       <c r="E549" s="22" t="inlineStr">
         <is>
-          <t>C20989</t>
+          <t>C25334</t>
         </is>
       </c>
       <c r="F549" s="21" t="inlineStr">
         <is>
-          <t>Vital Signs;Body Water Measurement</t>
+          <t>Vital Signs;Body Measurements</t>
         </is>
       </c>
       <c r="G549" s="20" t="inlineStr">
         <is>
-          <t>TBW;Total Body Water</t>
+          <t>BODLNGTH;Body Length</t>
         </is>
       </c>
       <c r="H549" s="20" t="inlineStr">
@@ -41436,7 +41436,7 @@
       </c>
       <c r="I549" s="21" t="inlineStr">
         <is>
-          <t>A measurement of the quantity of water within the body, including both the intracellular and extracellular compartments.</t>
+          <t>The total linear extent of the body.</t>
         </is>
       </c>
       <c r="J549" s="20" t="inlineStr"/>
@@ -41618,32 +41618,32 @@
       </c>
       <c r="B552" s="21" t="inlineStr">
         <is>
-          <t>Total Lung Capacity</t>
+          <t>Total Body Water Measurement</t>
         </is>
       </c>
       <c r="C552" s="20" t="inlineStr">
         <is>
-          <t>C111325</t>
+          <t>C104622</t>
         </is>
       </c>
       <c r="D552" s="22" t="inlineStr">
         <is>
-          <t>C111325</t>
+          <t>C104622</t>
         </is>
       </c>
       <c r="E552" s="22" t="inlineStr">
         <is>
-          <t>C38081</t>
+          <t>C20989</t>
         </is>
       </c>
       <c r="F552" s="21" t="inlineStr">
         <is>
-          <t>Respiratory System Findings;Pulmonary Function Test</t>
+          <t>Vital Signs;Body Water Measurement</t>
         </is>
       </c>
       <c r="G552" s="20" t="inlineStr">
         <is>
-          <t>Lung volume test;TLC;TLUNGCAP;Total lung capacity</t>
+          <t>TBW;Total Body Water</t>
         </is>
       </c>
       <c r="H552" s="20" t="inlineStr">
@@ -41653,49 +41653,33 @@
       </c>
       <c r="I552" s="21" t="inlineStr">
         <is>
-          <t>The total volume of air in the lungs after maximum inhalation.</t>
-        </is>
-      </c>
-      <c r="J552" s="20" t="inlineStr">
-        <is>
-          <t>http://loinc.org/</t>
-        </is>
-      </c>
-      <c r="K552" s="20" t="inlineStr">
-        <is>
-          <t>LOINC</t>
-        </is>
-      </c>
-      <c r="L552" s="20" t="inlineStr">
-        <is>
-          <t>19862-2</t>
-        </is>
-      </c>
+          <t>A measurement of the quantity of water within the body, including both the intracellular and extracellular compartments.</t>
+        </is>
+      </c>
+      <c r="J552" s="20" t="inlineStr"/>
+      <c r="K552" s="20" t="inlineStr"/>
+      <c r="L552" s="20" t="inlineStr"/>
       <c r="M552" s="20" t="inlineStr">
         <is>
-          <t>C44279</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="N552" s="22" t="inlineStr">
         <is>
-          <t>C44279</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="O552" s="20" t="inlineStr">
         <is>
-          <t>Unit of Volume</t>
+          <t>Observation Result</t>
         </is>
       </c>
       <c r="P552" s="20" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="Q552" s="21" t="inlineStr">
-        <is>
-          <t>mL;L</t>
-        </is>
-      </c>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="Q552" s="21" t="inlineStr"/>
     </row>
     <row r="553">
       <c r="A553" s="20" t="inlineStr">
@@ -41760,22 +41744,22 @@
       </c>
       <c r="M553" s="20" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="N553" s="22" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="O553" s="20" t="inlineStr">
         <is>
-          <t>Observation Result</t>
+          <t>Collection Date Time</t>
         </is>
       </c>
       <c r="P553" s="20" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="Q553" s="21" t="inlineStr"/>
@@ -41843,25 +41827,29 @@
       </c>
       <c r="M554" s="20" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C44279</t>
         </is>
       </c>
       <c r="N554" s="22" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C44279</t>
         </is>
       </c>
       <c r="O554" s="20" t="inlineStr">
         <is>
-          <t>Collection Date Time</t>
+          <t>Unit of Volume</t>
         </is>
       </c>
       <c r="P554" s="20" t="inlineStr">
         <is>
-          <t>datetime</t>
-        </is>
-      </c>
-      <c r="Q554" s="21" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="Q554" s="21" t="inlineStr">
+        <is>
+          <t>mL;L</t>
+        </is>
+      </c>
     </row>
     <row r="555">
       <c r="A555" s="20" t="inlineStr">
@@ -41871,17 +41859,17 @@
       </c>
       <c r="B555" s="21" t="inlineStr">
         <is>
-          <t>Total Respiratory System Resistance</t>
+          <t>Total Lung Capacity</t>
         </is>
       </c>
       <c r="C555" s="20" t="inlineStr">
         <is>
-          <t>C122185</t>
+          <t>C111325</t>
         </is>
       </c>
       <c r="D555" s="22" t="inlineStr">
         <is>
-          <t>C122185</t>
+          <t>C111325</t>
         </is>
       </c>
       <c r="E555" s="22" t="inlineStr">
@@ -41896,7 +41884,7 @@
       </c>
       <c r="G555" s="20" t="inlineStr">
         <is>
-          <t>RRS</t>
+          <t>Lung volume test;TLC;TLUNGCAP;Total lung capacity</t>
         </is>
       </c>
       <c r="H555" s="20" t="inlineStr">
@@ -41906,30 +41894,42 @@
       </c>
       <c r="I555" s="21" t="inlineStr">
         <is>
-          <t>A calculated value based on all factors that influence the flow of gas from the airway opening to the alveoli, including airway resistance, and tissue resistance of the lung and chest wall.</t>
-        </is>
-      </c>
-      <c r="J555" s="20" t="inlineStr"/>
-      <c r="K555" s="20" t="inlineStr"/>
-      <c r="L555" s="20" t="inlineStr"/>
+          <t>The total volume of air in the lungs after maximum inhalation.</t>
+        </is>
+      </c>
+      <c r="J555" s="20" t="inlineStr">
+        <is>
+          <t>http://loinc.org/</t>
+        </is>
+      </c>
+      <c r="K555" s="20" t="inlineStr">
+        <is>
+          <t>LOINC</t>
+        </is>
+      </c>
+      <c r="L555" s="20" t="inlineStr">
+        <is>
+          <t>19862-2</t>
+        </is>
+      </c>
       <c r="M555" s="20" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="N555" s="22" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="O555" s="20" t="inlineStr">
         <is>
-          <t>Collection Date Time</t>
+          <t>Observation Result</t>
         </is>
       </c>
       <c r="P555" s="20" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="Q555" s="21" t="inlineStr"/>
@@ -41985,29 +41985,25 @@
       <c r="L556" s="20" t="inlineStr"/>
       <c r="M556" s="20" t="inlineStr">
         <is>
-          <t>C67332</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="N556" s="22" t="inlineStr">
         <is>
-          <t>C67332</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="O556" s="20" t="inlineStr">
         <is>
-          <t>Manometric Unit of Pressure</t>
+          <t>Observation Result</t>
         </is>
       </c>
       <c r="P556" s="20" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="Q556" s="21" t="inlineStr">
-        <is>
-          <t>cmH2O*s/mL</t>
-        </is>
-      </c>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="Q556" s="21" t="inlineStr"/>
     </row>
     <row r="557">
       <c r="A557" s="20" t="inlineStr">
@@ -42060,25 +42056,29 @@
       <c r="L557" s="20" t="inlineStr"/>
       <c r="M557" s="20" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C67332</t>
         </is>
       </c>
       <c r="N557" s="22" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C67332</t>
         </is>
       </c>
       <c r="O557" s="20" t="inlineStr">
         <is>
-          <t>Observation Result</t>
+          <t>Manometric Unit of Pressure</t>
         </is>
       </c>
       <c r="P557" s="20" t="inlineStr">
         <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="Q557" s="21" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="Q557" s="21" t="inlineStr">
+        <is>
+          <t>cmH2O*s/mL</t>
+        </is>
+      </c>
     </row>
     <row r="558">
       <c r="A558" s="20" t="inlineStr">
@@ -42088,32 +42088,32 @@
       </c>
       <c r="B558" s="21" t="inlineStr">
         <is>
-          <t>Triceps Skinfold Thickness</t>
+          <t>Total Respiratory System Resistance</t>
         </is>
       </c>
       <c r="C558" s="20" t="inlineStr">
         <is>
-          <t>C98793</t>
+          <t>C122185</t>
         </is>
       </c>
       <c r="D558" s="22" t="inlineStr">
         <is>
-          <t>C98793</t>
+          <t>C122185</t>
         </is>
       </c>
       <c r="E558" s="22" t="inlineStr">
         <is>
-          <t>C77537</t>
+          <t>C38081</t>
         </is>
       </c>
       <c r="F558" s="21" t="inlineStr">
         <is>
-          <t>Vital Signs;Body Measurements</t>
+          <t>Respiratory System Findings;Pulmonary Function Test</t>
         </is>
       </c>
       <c r="G558" s="20" t="inlineStr">
         <is>
-          <t>TRSKNF</t>
+          <t>RRS</t>
         </is>
       </c>
       <c r="H558" s="20" t="inlineStr">
@@ -42123,42 +42123,30 @@
       </c>
       <c r="I558" s="21" t="inlineStr">
         <is>
-          <t>A measurement of the thickness of a pinch of skin on the triceps.</t>
-        </is>
-      </c>
-      <c r="J558" s="20" t="inlineStr">
-        <is>
-          <t>http://loinc.org/</t>
-        </is>
-      </c>
-      <c r="K558" s="20" t="inlineStr">
-        <is>
-          <t>LOINC</t>
-        </is>
-      </c>
-      <c r="L558" s="20" t="inlineStr">
-        <is>
-          <t>8354-3</t>
-        </is>
-      </c>
+          <t>A calculated value based on all factors that influence the flow of gas from the airway opening to the alveoli, including airway resistance, and tissue resistance of the lung and chest wall.</t>
+        </is>
+      </c>
+      <c r="J558" s="20" t="inlineStr"/>
+      <c r="K558" s="20" t="inlineStr"/>
+      <c r="L558" s="20" t="inlineStr"/>
       <c r="M558" s="20" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="N558" s="22" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="O558" s="20" t="inlineStr">
         <is>
-          <t>Observation Result</t>
+          <t>Collection Date Time</t>
         </is>
       </c>
       <c r="P558" s="20" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="Q558" s="21" t="inlineStr"/>
@@ -42226,29 +42214,25 @@
       </c>
       <c r="M559" s="20" t="inlineStr">
         <is>
-          <t>C42578</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="N559" s="22" t="inlineStr">
         <is>
-          <t>C42578</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="O559" s="20" t="inlineStr">
         <is>
-          <t>Unit of Length</t>
+          <t>Observation Result</t>
         </is>
       </c>
       <c r="P559" s="20" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="Q559" s="21" t="inlineStr">
-        <is>
-          <t>mm;cm;in</t>
-        </is>
-      </c>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="Q559" s="21" t="inlineStr"/>
     </row>
     <row r="560">
       <c r="A560" s="20" t="inlineStr">
@@ -42313,25 +42297,29 @@
       </c>
       <c r="M560" s="20" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C42578</t>
         </is>
       </c>
       <c r="N560" s="22" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C42578</t>
         </is>
       </c>
       <c r="O560" s="20" t="inlineStr">
         <is>
-          <t>Collection Date Time</t>
+          <t>Unit of Length</t>
         </is>
       </c>
       <c r="P560" s="20" t="inlineStr">
         <is>
-          <t>datetime</t>
-        </is>
-      </c>
-      <c r="Q560" s="21" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="Q560" s="21" t="inlineStr">
+        <is>
+          <t>mm;cm;in</t>
+        </is>
+      </c>
     </row>
     <row r="561">
       <c r="A561" s="20" t="inlineStr">
@@ -42341,22 +42329,22 @@
       </c>
       <c r="B561" s="21" t="inlineStr">
         <is>
-          <t>Ulnar Length</t>
+          <t>Triceps Skinfold Thickness</t>
         </is>
       </c>
       <c r="C561" s="20" t="inlineStr">
         <is>
-          <t>C174376</t>
+          <t>C98793</t>
         </is>
       </c>
       <c r="D561" s="22" t="inlineStr">
         <is>
-          <t>C174376</t>
+          <t>C98793</t>
         </is>
       </c>
       <c r="E561" s="22" t="inlineStr">
         <is>
-          <t>C25334</t>
+          <t>C77537</t>
         </is>
       </c>
       <c r="F561" s="21" t="inlineStr">
@@ -42366,7 +42354,7 @@
       </c>
       <c r="G561" s="20" t="inlineStr">
         <is>
-          <t>ULNARL</t>
+          <t>TRSKNF</t>
         </is>
       </c>
       <c r="H561" s="20" t="inlineStr">
@@ -42376,12 +42364,24 @@
       </c>
       <c r="I561" s="21" t="inlineStr">
         <is>
-          <t>A measurement of the length of the ulna.</t>
-        </is>
-      </c>
-      <c r="J561" s="20" t="inlineStr"/>
-      <c r="K561" s="20" t="inlineStr"/>
-      <c r="L561" s="20" t="inlineStr"/>
+          <t>A measurement of the thickness of a pinch of skin on the triceps.</t>
+        </is>
+      </c>
+      <c r="J561" s="20" t="inlineStr">
+        <is>
+          <t>http://loinc.org/</t>
+        </is>
+      </c>
+      <c r="K561" s="20" t="inlineStr">
+        <is>
+          <t>LOINC</t>
+        </is>
+      </c>
+      <c r="L561" s="20" t="inlineStr">
+        <is>
+          <t>8354-3</t>
+        </is>
+      </c>
       <c r="M561" s="20" t="inlineStr">
         <is>
           <t>C82515</t>
@@ -42455,22 +42455,22 @@
       <c r="L562" s="20" t="inlineStr"/>
       <c r="M562" s="20" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="N562" s="22" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="O562" s="20" t="inlineStr">
         <is>
-          <t>Observation Result</t>
+          <t>Collection Date Time</t>
         </is>
       </c>
       <c r="P562" s="20" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="Q562" s="21" t="inlineStr"/>
@@ -42526,29 +42526,25 @@
       <c r="L563" s="20" t="inlineStr"/>
       <c r="M563" s="20" t="inlineStr">
         <is>
-          <t>C42578</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="N563" s="22" t="inlineStr">
         <is>
-          <t>C42578</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="O563" s="20" t="inlineStr">
         <is>
-          <t>Unit of Length</t>
+          <t>Observation Result</t>
         </is>
       </c>
       <c r="P563" s="20" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="Q563" s="21" t="inlineStr">
-        <is>
-          <t>mm;cm;in</t>
-        </is>
-      </c>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="Q563" s="21" t="inlineStr"/>
     </row>
     <row r="564">
       <c r="A564" s="20" t="inlineStr">
@@ -42558,40 +42554,72 @@
       </c>
       <c r="B564" s="21" t="inlineStr">
         <is>
-          <t>Ventilatory Threshold</t>
+          <t>Ulnar Length</t>
         </is>
       </c>
       <c r="C564" s="20" t="inlineStr">
         <is>
-          <t>C123909</t>
+          <t>C174376</t>
         </is>
       </c>
       <c r="D564" s="22" t="inlineStr">
         <is>
-          <t>C123909</t>
-        </is>
-      </c>
-      <c r="E564" s="20" t="n"/>
+          <t>C174376</t>
+        </is>
+      </c>
+      <c r="E564" s="22" t="inlineStr">
+        <is>
+          <t>C25334</t>
+        </is>
+      </c>
       <c r="F564" s="21" t="inlineStr">
         <is>
-          <t>Respiratory System Findings</t>
-        </is>
-      </c>
-      <c r="G564" s="20" t="inlineStr"/>
-      <c r="H564" s="20" t="inlineStr"/>
+          <t>Vital Signs;Body Measurements</t>
+        </is>
+      </c>
+      <c r="G564" s="20" t="inlineStr">
+        <is>
+          <t>ULNARL</t>
+        </is>
+      </c>
+      <c r="H564" s="20" t="inlineStr">
+        <is>
+          <t>Quantitative</t>
+        </is>
+      </c>
       <c r="I564" s="21" t="inlineStr">
         <is>
-          <t>The point during exercise at which pulmonary ventilation becomes disproportionately high with respect to oxygen consumption.</t>
+          <t>A measurement of the length of the ulna.</t>
         </is>
       </c>
       <c r="J564" s="20" t="inlineStr"/>
       <c r="K564" s="20" t="inlineStr"/>
       <c r="L564" s="20" t="inlineStr"/>
-      <c r="M564" s="20" t="inlineStr"/>
-      <c r="N564" s="20" t="n"/>
-      <c r="O564" s="20" t="inlineStr"/>
-      <c r="P564" s="20" t="inlineStr"/>
-      <c r="Q564" s="21" t="inlineStr"/>
+      <c r="M564" s="20" t="inlineStr">
+        <is>
+          <t>C42578</t>
+        </is>
+      </c>
+      <c r="N564" s="22" t="inlineStr">
+        <is>
+          <t>C42578</t>
+        </is>
+      </c>
+      <c r="O564" s="20" t="inlineStr">
+        <is>
+          <t>Unit of Length</t>
+        </is>
+      </c>
+      <c r="P564" s="20" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="Q564" s="21" t="inlineStr">
+        <is>
+          <t>mm;cm;in</t>
+        </is>
+      </c>
     </row>
     <row r="565">
       <c r="A565" s="20" t="inlineStr">
@@ -42601,17 +42629,17 @@
       </c>
       <c r="B565" s="21" t="inlineStr">
         <is>
-          <t>Volume</t>
+          <t>Ventilatory Threshold</t>
         </is>
       </c>
       <c r="C565" s="20" t="inlineStr">
         <is>
-          <t>C25335</t>
+          <t>C123909</t>
         </is>
       </c>
       <c r="D565" s="22" t="inlineStr">
         <is>
-          <t>C25335</t>
+          <t>C123909</t>
         </is>
       </c>
       <c r="E565" s="20" t="n"/>
@@ -42620,15 +42648,11 @@
           <t>Respiratory System Findings</t>
         </is>
       </c>
-      <c r="G565" s="20" t="inlineStr">
-        <is>
-          <t>Vol;Total Volume</t>
-        </is>
-      </c>
+      <c r="G565" s="20" t="inlineStr"/>
       <c r="H565" s="20" t="inlineStr"/>
       <c r="I565" s="21" t="inlineStr">
         <is>
-          <t>The amount of three dimensional space occupied by an object or the capacity of a space or container.</t>
+          <t>The point during exercise at which pulmonary ventilation becomes disproportionately high with respect to oxygen consumption.</t>
         </is>
       </c>
       <c r="J565" s="20" t="inlineStr"/>
@@ -42648,17 +42672,17 @@
       </c>
       <c r="B566" s="21" t="inlineStr">
         <is>
-          <t>Volume Measurement</t>
+          <t>Volume</t>
         </is>
       </c>
       <c r="C566" s="20" t="inlineStr">
         <is>
-          <t>C74720</t>
+          <t>C25335</t>
         </is>
       </c>
       <c r="D566" s="22" t="inlineStr">
         <is>
-          <t>C74720</t>
+          <t>C25335</t>
         </is>
       </c>
       <c r="E566" s="20" t="n"/>
@@ -42669,13 +42693,13 @@
       </c>
       <c r="G566" s="20" t="inlineStr">
         <is>
-          <t>VOL;VOLUME;Volume</t>
+          <t>Vol;Total Volume</t>
         </is>
       </c>
       <c r="H566" s="20" t="inlineStr"/>
       <c r="I566" s="21" t="inlineStr">
         <is>
-          <t>The determination of the volume of a sample.</t>
+          <t>The amount of three dimensional space occupied by an object or the capacity of a space or container.</t>
         </is>
       </c>
       <c r="J566" s="20" t="inlineStr"/>
@@ -42695,67 +42719,43 @@
       </c>
       <c r="B567" s="21" t="inlineStr">
         <is>
-          <t>Waist to Heel Length</t>
+          <t>Volume Measurement</t>
         </is>
       </c>
       <c r="C567" s="20" t="inlineStr">
         <is>
-          <t>C181552</t>
+          <t>C74720</t>
         </is>
       </c>
       <c r="D567" s="22" t="inlineStr">
         <is>
-          <t>C181552</t>
-        </is>
-      </c>
-      <c r="E567" s="22" t="inlineStr">
-        <is>
-          <t>C25334</t>
-        </is>
-      </c>
+          <t>C74720</t>
+        </is>
+      </c>
+      <c r="E567" s="20" t="n"/>
       <c r="F567" s="21" t="inlineStr">
         <is>
-          <t>Vital Signs;Body Measurements</t>
+          <t>Respiratory System Findings</t>
         </is>
       </c>
       <c r="G567" s="20" t="inlineStr">
         <is>
-          <t>WASTHEEL</t>
-        </is>
-      </c>
-      <c r="H567" s="20" t="inlineStr">
-        <is>
-          <t>Quantitative</t>
-        </is>
-      </c>
+          <t>VOL;VOLUME;Volume</t>
+        </is>
+      </c>
+      <c r="H567" s="20" t="inlineStr"/>
       <c r="I567" s="21" t="inlineStr">
         <is>
-          <t>A measurement from the top of the waist to the bottom of the heel.</t>
+          <t>The determination of the volume of a sample.</t>
         </is>
       </c>
       <c r="J567" s="20" t="inlineStr"/>
       <c r="K567" s="20" t="inlineStr"/>
       <c r="L567" s="20" t="inlineStr"/>
-      <c r="M567" s="20" t="inlineStr">
-        <is>
-          <t>C70856</t>
-        </is>
-      </c>
-      <c r="N567" s="22" t="inlineStr">
-        <is>
-          <t>C70856</t>
-        </is>
-      </c>
-      <c r="O567" s="20" t="inlineStr">
-        <is>
-          <t>Observation Result</t>
-        </is>
-      </c>
-      <c r="P567" s="20" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
+      <c r="M567" s="20" t="inlineStr"/>
+      <c r="N567" s="20" t="n"/>
+      <c r="O567" s="20" t="inlineStr"/>
+      <c r="P567" s="20" t="inlineStr"/>
       <c r="Q567" s="21" t="inlineStr"/>
     </row>
     <row r="568">
@@ -42809,29 +42809,25 @@
       <c r="L568" s="20" t="inlineStr"/>
       <c r="M568" s="20" t="inlineStr">
         <is>
-          <t>C42578</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="N568" s="22" t="inlineStr">
         <is>
-          <t>C42578</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="O568" s="20" t="inlineStr">
         <is>
-          <t>Unit of Length</t>
+          <t>Collection Date Time</t>
         </is>
       </c>
       <c r="P568" s="20" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="Q568" s="21" t="inlineStr">
-        <is>
-          <t>mm;cm;in;ft</t>
-        </is>
-      </c>
+          <t>datetime</t>
+        </is>
+      </c>
+      <c r="Q568" s="21" t="inlineStr"/>
     </row>
     <row r="569">
       <c r="A569" s="20" t="inlineStr">
@@ -42884,25 +42880,29 @@
       <c r="L569" s="20" t="inlineStr"/>
       <c r="M569" s="20" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C42578</t>
         </is>
       </c>
       <c r="N569" s="22" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C42578</t>
         </is>
       </c>
       <c r="O569" s="20" t="inlineStr">
         <is>
-          <t>Collection Date Time</t>
+          <t>Unit of Length</t>
         </is>
       </c>
       <c r="P569" s="20" t="inlineStr">
         <is>
-          <t>datetime</t>
-        </is>
-      </c>
-      <c r="Q569" s="21" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="Q569" s="21" t="inlineStr">
+        <is>
+          <t>mm;cm;in;ft</t>
+        </is>
+      </c>
     </row>
     <row r="570">
       <c r="A570" s="20" t="inlineStr">
@@ -42912,22 +42912,22 @@
       </c>
       <c r="B570" s="21" t="inlineStr">
         <is>
-          <t>Waist-Hip Ratio</t>
+          <t>Waist to Heel Length</t>
         </is>
       </c>
       <c r="C570" s="20" t="inlineStr">
         <is>
-          <t>C17651</t>
+          <t>C181552</t>
         </is>
       </c>
       <c r="D570" s="22" t="inlineStr">
         <is>
-          <t>C17651</t>
+          <t>C181552</t>
         </is>
       </c>
       <c r="E570" s="22" t="inlineStr">
         <is>
-          <t>C19332</t>
+          <t>C25334</t>
         </is>
       </c>
       <c r="F570" s="21" t="inlineStr">
@@ -42937,7 +42937,7 @@
       </c>
       <c r="G570" s="20" t="inlineStr">
         <is>
-          <t>Waist to Hip Ratio;WAISTHIP</t>
+          <t>WASTHEEL</t>
         </is>
       </c>
       <c r="H570" s="20" t="inlineStr">
@@ -42947,7 +42947,7 @@
       </c>
       <c r="I570" s="21" t="inlineStr">
         <is>
-          <t>The ratio of the abdominal circumference at the navel to maximum hip and buttocks circumference; looks at the proportion of fat stored on the body around the waist and hip. Carrying extra weight around the waist is a greater health risk than carrying extra weight around the hips or thighs.</t>
+          <t>A measurement from the top of the waist to the bottom of the heel.</t>
         </is>
       </c>
       <c r="J570" s="20" t="inlineStr"/>
@@ -42955,29 +42955,25 @@
       <c r="L570" s="20" t="inlineStr"/>
       <c r="M570" s="20" t="inlineStr">
         <is>
-          <t>C48570</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="N570" s="22" t="inlineStr">
         <is>
-          <t>C48570</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="O570" s="20" t="inlineStr">
         <is>
-          <t>Percent Unit</t>
+          <t>Observation Result</t>
         </is>
       </c>
       <c r="P570" s="20" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="Q570" s="21" t="inlineStr">
-        <is>
-          <t>RATIO</t>
-        </is>
-      </c>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="Q570" s="21" t="inlineStr"/>
     </row>
     <row r="571">
       <c r="A571" s="20" t="inlineStr">
@@ -43030,22 +43026,22 @@
       <c r="L571" s="20" t="inlineStr"/>
       <c r="M571" s="20" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="N571" s="22" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="O571" s="20" t="inlineStr">
         <is>
-          <t>Collection Date Time</t>
+          <t>Observation Result</t>
         </is>
       </c>
       <c r="P571" s="20" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="Q571" s="21" t="inlineStr"/>
@@ -43101,25 +43097,29 @@
       <c r="L572" s="20" t="inlineStr"/>
       <c r="M572" s="20" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C48570</t>
         </is>
       </c>
       <c r="N572" s="22" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C48570</t>
         </is>
       </c>
       <c r="O572" s="20" t="inlineStr">
         <is>
-          <t>Observation Result</t>
+          <t>Percent Unit</t>
         </is>
       </c>
       <c r="P572" s="20" t="inlineStr">
         <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="Q572" s="21" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="Q572" s="21" t="inlineStr">
+        <is>
+          <t>RATIO</t>
+        </is>
+      </c>
     </row>
     <row r="573">
       <c r="A573" s="20" t="inlineStr">
@@ -43129,20 +43129,24 @@
       </c>
       <c r="B573" s="21" t="inlineStr">
         <is>
-          <t>Weight-for-Age Percentile</t>
+          <t>Waist-Hip Ratio</t>
         </is>
       </c>
       <c r="C573" s="20" t="inlineStr">
         <is>
-          <t>C163569</t>
+          <t>C17651</t>
         </is>
       </c>
       <c r="D573" s="22" t="inlineStr">
         <is>
-          <t>C163569</t>
-        </is>
-      </c>
-      <c r="E573" s="20" t="n"/>
+          <t>C17651</t>
+        </is>
+      </c>
+      <c r="E573" s="22" t="inlineStr">
+        <is>
+          <t>C19332</t>
+        </is>
+      </c>
       <c r="F573" s="21" t="inlineStr">
         <is>
           <t>Vital Signs;Body Measurements</t>
@@ -43150,7 +43154,7 @@
       </c>
       <c r="G573" s="20" t="inlineStr">
         <is>
-          <t>WTAPCTL</t>
+          <t>Waist to Hip Ratio;WAISTHIP</t>
         </is>
       </c>
       <c r="H573" s="20" t="inlineStr">
@@ -43160,24 +43164,12 @@
       </c>
       <c r="I573" s="21" t="inlineStr">
         <is>
-          <t>A measurement of an individual's weight in relationship to age, in comparison to a reference percentile curve.</t>
-        </is>
-      </c>
-      <c r="J573" s="20" t="inlineStr">
-        <is>
-          <t>http://loinc.org/</t>
-        </is>
-      </c>
-      <c r="K573" s="20" t="inlineStr">
-        <is>
-          <t>LOINC</t>
-        </is>
-      </c>
-      <c r="L573" s="20" t="inlineStr">
-        <is>
-          <t>8336-0</t>
-        </is>
-      </c>
+          <t>The ratio of the abdominal circumference at the navel to maximum hip and buttocks circumference; looks at the proportion of fat stored on the body around the waist and hip. Carrying extra weight around the waist is a greater health risk than carrying extra weight around the hips or thighs.</t>
+        </is>
+      </c>
+      <c r="J573" s="20" t="inlineStr"/>
+      <c r="K573" s="20" t="inlineStr"/>
+      <c r="L573" s="20" t="inlineStr"/>
       <c r="M573" s="20" t="inlineStr">
         <is>
           <t>C82515</t>
@@ -43259,22 +43251,22 @@
       </c>
       <c r="M574" s="20" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="N574" s="22" t="inlineStr">
         <is>
-          <t>C70856</t>
+          <t>C82515</t>
         </is>
       </c>
       <c r="O574" s="20" t="inlineStr">
         <is>
-          <t>Observation Result</t>
+          <t>Collection Date Time</t>
         </is>
       </c>
       <c r="P574" s="20" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="Q574" s="21" t="inlineStr"/>
@@ -43287,17 +43279,17 @@
       </c>
       <c r="B575" s="21" t="inlineStr">
         <is>
-          <t>Weight-for-Height Percentile</t>
+          <t>Weight-for-Age Percentile</t>
         </is>
       </c>
       <c r="C575" s="20" t="inlineStr">
         <is>
-          <t>C163570</t>
+          <t>C163569</t>
         </is>
       </c>
       <c r="D575" s="22" t="inlineStr">
         <is>
-          <t>C163570</t>
+          <t>C163569</t>
         </is>
       </c>
       <c r="E575" s="20" t="n"/>
@@ -43308,7 +43300,7 @@
       </c>
       <c r="G575" s="20" t="inlineStr">
         <is>
-          <t>WTHTPCTL</t>
+          <t>WTAPCTL</t>
         </is>
       </c>
       <c r="H575" s="20" t="inlineStr">
@@ -43318,30 +43310,42 @@
       </c>
       <c r="I575" s="21" t="inlineStr">
         <is>
-          <t>A measurement of an individual's weight in relationship to height, in comparison to a reference percentile curve.</t>
-        </is>
-      </c>
-      <c r="J575" s="20" t="inlineStr"/>
-      <c r="K575" s="20" t="inlineStr"/>
-      <c r="L575" s="20" t="inlineStr"/>
+          <t>A measurement of an individual's weight in relationship to age, in comparison to a reference percentile curve.</t>
+        </is>
+      </c>
+      <c r="J575" s="20" t="inlineStr">
+        <is>
+          <t>http://loinc.org/</t>
+        </is>
+      </c>
+      <c r="K575" s="20" t="inlineStr">
+        <is>
+          <t>LOINC</t>
+        </is>
+      </c>
+      <c r="L575" s="20" t="inlineStr">
+        <is>
+          <t>8336-0</t>
+        </is>
+      </c>
       <c r="M575" s="20" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="N575" s="22" t="inlineStr">
         <is>
-          <t>C82515</t>
+          <t>C70856</t>
         </is>
       </c>
       <c r="O575" s="20" t="inlineStr">
         <is>
-          <t>Collection Date Time</t>
+          <t>Observation Result</t>
         </is>
       </c>
       <c r="P575" s="20" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="Q575" s="21" t="inlineStr"/>
@@ -43413,8 +43417,75 @@
       </c>
       <c r="Q576" s="21" t="inlineStr"/>
     </row>
+    <row r="577">
+      <c r="A577" s="20" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B577" s="21" t="inlineStr">
+        <is>
+          <t>Weight-for-Height Percentile</t>
+        </is>
+      </c>
+      <c r="C577" s="20" t="inlineStr">
+        <is>
+          <t>C163570</t>
+        </is>
+      </c>
+      <c r="D577" s="22" t="inlineStr">
+        <is>
+          <t>C163570</t>
+        </is>
+      </c>
+      <c r="E577" s="20" t="n"/>
+      <c r="F577" s="21" t="inlineStr">
+        <is>
+          <t>Vital Signs;Body Measurements</t>
+        </is>
+      </c>
+      <c r="G577" s="20" t="inlineStr">
+        <is>
+          <t>WTHTPCTL</t>
+        </is>
+      </c>
+      <c r="H577" s="20" t="inlineStr">
+        <is>
+          <t>Quantitative</t>
+        </is>
+      </c>
+      <c r="I577" s="21" t="inlineStr">
+        <is>
+          <t>A measurement of an individual's weight in relationship to height, in comparison to a reference percentile curve.</t>
+        </is>
+      </c>
+      <c r="J577" s="20" t="inlineStr"/>
+      <c r="K577" s="20" t="inlineStr"/>
+      <c r="L577" s="20" t="inlineStr"/>
+      <c r="M577" s="20" t="inlineStr">
+        <is>
+          <t>C82515</t>
+        </is>
+      </c>
+      <c r="N577" s="22" t="inlineStr">
+        <is>
+          <t>C82515</t>
+        </is>
+      </c>
+      <c r="O577" s="20" t="inlineStr">
+        <is>
+          <t>Collection Date Time</t>
+        </is>
+      </c>
+      <c r="P577" s="20" t="inlineStr">
+        <is>
+          <t>datetime</t>
+        </is>
+      </c>
+      <c r="Q577" s="21" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q576"/>
+  <autoFilter ref="A1:Q577"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -44793,9 +44864,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E478" r:id="rId1375"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N478" r:id="rId1376"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D479" r:id="rId1377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D480" r:id="rId1378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E480" r:id="rId1379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N480" r:id="rId1380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E479" r:id="rId1378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N479" r:id="rId1379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D480" r:id="rId1380"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D481" r:id="rId1381"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E481" r:id="rId1382"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N481" r:id="rId1383"/>
@@ -44851,9 +44922,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E498" r:id="rId1433"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N498" r:id="rId1434"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D499" r:id="rId1435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D500" r:id="rId1436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E500" r:id="rId1437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N500" r:id="rId1438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E499" r:id="rId1436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N499" r:id="rId1437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D500" r:id="rId1438"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D501" r:id="rId1439"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E501" r:id="rId1440"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N501" r:id="rId1441"/>
@@ -44888,9 +44959,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E511" r:id="rId1470"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N511" r:id="rId1471"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D512" r:id="rId1472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D513" r:id="rId1473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E513" r:id="rId1474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N513" r:id="rId1475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E512" r:id="rId1473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N512" r:id="rId1474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D513" r:id="rId1475"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D514" r:id="rId1476"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E514" r:id="rId1477"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N514" r:id="rId1478"/>
@@ -44931,16 +45002,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E526" r:id="rId1513"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N526" r:id="rId1514"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D527" r:id="rId1515"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D528" r:id="rId1516"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N528" r:id="rId1517"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D529" r:id="rId1518"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N529" r:id="rId1519"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D530" r:id="rId1520"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N530" r:id="rId1521"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D531" r:id="rId1522"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N531" r:id="rId1523"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D532" r:id="rId1524"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E532" r:id="rId1525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E527" r:id="rId1516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N527" r:id="rId1517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D528" r:id="rId1518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D529" r:id="rId1519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N529" r:id="rId1520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D530" r:id="rId1521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N530" r:id="rId1522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D531" r:id="rId1523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N531" r:id="rId1524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D532" r:id="rId1525"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N532" r:id="rId1526"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D533" r:id="rId1527"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E533" r:id="rId1528"/>
@@ -45036,11 +45107,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E563" r:id="rId1618"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N563" r:id="rId1619"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D564" r:id="rId1620"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D565" r:id="rId1621"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D566" r:id="rId1622"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D567" r:id="rId1623"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E567" r:id="rId1624"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N567" r:id="rId1625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E564" r:id="rId1621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N564" r:id="rId1622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D565" r:id="rId1623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D566" r:id="rId1624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D567" r:id="rId1625"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D568" r:id="rId1626"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E568" r:id="rId1627"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N568" r:id="rId1628"/>
@@ -45057,13 +45128,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E572" r:id="rId1639"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N572" r:id="rId1640"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D573" r:id="rId1641"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N573" r:id="rId1642"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D574" r:id="rId1643"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N574" r:id="rId1644"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D575" r:id="rId1645"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N575" r:id="rId1646"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D576" r:id="rId1647"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N576" r:id="rId1648"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E573" r:id="rId1642"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N573" r:id="rId1643"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D574" r:id="rId1644"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N574" r:id="rId1645"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D575" r:id="rId1646"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N575" r:id="rId1647"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D576" r:id="rId1648"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N576" r:id="rId1649"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D577" r:id="rId1650"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N577" r:id="rId1651"/>
   </hyperlinks>
   <pageMargins left="0.05" right="0.05" top="0.5" bottom="0.5" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -54874,7 +54948,7 @@
         </is>
       </c>
       <c r="K181" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="182">

</xml_diff>